<commit_message>
Update company radar data
</commit_message>
<xml_diff>
--- a/company_radar_output.xlsx
+++ b/company_radar_output.xlsx
@@ -876,13 +876,13 @@
         <v>1.694015495883381</v>
       </c>
       <c r="AW2" t="n">
-        <v>2.255401252426652</v>
+        <v>2.255400839571528</v>
       </c>
       <c r="AX2" t="n">
         <v>1.563350686211098</v>
       </c>
       <c r="AY2" t="n">
-        <v>3.052599355162004</v>
+        <v>3.052598715344739</v>
       </c>
       <c r="AZ2" t="inlineStr"/>
       <c r="BA2" t="n">
@@ -1216,16 +1216,16 @@
         <v>372.6216882324219</v>
       </c>
       <c r="AG4" t="n">
-        <v>318.5789504241943</v>
+        <v>318.578950881958</v>
       </c>
       <c r="AH4" t="n">
         <v>-0.04144067842612775</v>
       </c>
       <c r="AI4" t="n">
-        <v>0.1211663300421728</v>
+        <v>0.1211663284311773</v>
       </c>
       <c r="AJ4" t="n">
-        <v>0.1696368756826796</v>
+        <v>0.1696368740020371</v>
       </c>
       <c r="AK4" t="n">
         <v>402.3796691894531</v>
@@ -1264,13 +1264,13 @@
         <v>1.016658868474406</v>
       </c>
       <c r="AW4" t="n">
-        <v>1.876851136246393</v>
+        <v>1.876851313028276</v>
       </c>
       <c r="AX4" t="n">
-        <v>0.1348402579903003</v>
+        <v>0.1348403680257064</v>
       </c>
       <c r="AY4" t="n">
-        <v>142.5068301988223</v>
+        <v>142.5068439455128</v>
       </c>
       <c r="AZ4" t="inlineStr"/>
       <c r="BA4" t="n">
@@ -1602,25 +1602,25 @@
         <v>600.0849096679688</v>
       </c>
       <c r="AG6" t="n">
-        <v>641.6731106567382</v>
+        <v>641.6731109619141</v>
       </c>
       <c r="AH6" t="n">
         <v>0.1151922189527061</v>
       </c>
       <c r="AI6" t="n">
-        <v>0.04291423601611521</v>
+        <v>0.04291423552011153</v>
       </c>
       <c r="AJ6" t="n">
-        <v>-0.06481212988059426</v>
+        <v>-0.06481213032536393</v>
       </c>
       <c r="AK6" t="n">
-        <v>787.419189453125</v>
+        <v>787.4192504882812</v>
       </c>
       <c r="AL6" t="n">
         <v>525.233154296875</v>
       </c>
       <c r="AM6" t="n">
-        <v>-0.1501222843737995</v>
+        <v>-0.1501223502502931</v>
       </c>
       <c r="AN6" t="n">
         <v>0.2741199151232596</v>
@@ -1650,13 +1650,13 @@
         <v>-0.07677876083840129</v>
       </c>
       <c r="AW6" t="n">
-        <v>0.9032612657010106</v>
+        <v>0.9032607701303479</v>
       </c>
       <c r="AX6" t="n">
         <v>0.03074029207672369</v>
       </c>
       <c r="AY6" t="n">
-        <v>16.65856039000963</v>
+        <v>16.65855861251545</v>
       </c>
       <c r="AZ6" t="inlineStr"/>
       <c r="BA6" t="n">
@@ -2188,16 +2188,16 @@
         <v>182.4422756958008</v>
       </c>
       <c r="AG9" t="n">
-        <v>194.303373260498</v>
+        <v>194.3033737945557</v>
       </c>
       <c r="AH9" t="n">
         <v>-0.229126040807846</v>
       </c>
       <c r="AI9" t="n">
-        <v>-0.2761834391773752</v>
+        <v>-0.2761834411668401</v>
       </c>
       <c r="AJ9" t="n">
-        <v>-0.06104421845932317</v>
+        <v>-0.06104422104011464</v>
       </c>
       <c r="AK9" t="n">
         <v>324.6299743652344</v>
@@ -2236,13 +2236,13 @@
         <v>-0.3947107724147052</v>
       </c>
       <c r="AW9" t="n">
-        <v>0.8455305870177687</v>
+        <v>0.8455313260848825</v>
       </c>
       <c r="AX9" t="n">
-        <v>-0.2744543460752883</v>
+        <v>-0.2744542889615302</v>
       </c>
       <c r="AY9" t="n">
-        <v>2798.49658486407</v>
+        <v>2798.495962087439</v>
       </c>
       <c r="AZ9" t="inlineStr"/>
       <c r="BA9" t="n">
@@ -2576,16 +2576,16 @@
         <v>403.3287658691406</v>
       </c>
       <c r="AG11" t="n">
-        <v>440.7076475524902</v>
+        <v>440.7076486206055</v>
       </c>
       <c r="AH11" t="n">
         <v>-0.04519578395640467</v>
       </c>
       <c r="AI11" t="n">
-        <v>-0.1261780723747289</v>
+        <v>-0.1261780744925558</v>
       </c>
       <c r="AJ11" t="n">
-        <v>-0.08481559576044717</v>
+        <v>-0.08481559797852167</v>
       </c>
       <c r="AK11" t="n">
         <v>538.6585693359375</v>
@@ -2624,13 +2624,13 @@
         <v>-0.2259391799221225</v>
       </c>
       <c r="AW11" t="n">
-        <v>0.4452462928430114</v>
+        <v>0.4452464583667617</v>
       </c>
       <c r="AX11" t="n">
         <v>-0.1821056233913793</v>
       </c>
       <c r="AY11" t="n">
-        <v>6512.280083309905</v>
+        <v>6512.282135210159</v>
       </c>
       <c r="AZ11" t="inlineStr"/>
       <c r="BA11" t="n">
@@ -2822,7 +2822,7 @@
         <v>-0.2527098486195496</v>
       </c>
       <c r="AY12" t="n">
-        <v>653.3522551915103</v>
+        <v>653.3523106485549</v>
       </c>
       <c r="AZ12" t="inlineStr"/>
       <c r="BA12" t="n">
@@ -3008,13 +3008,13 @@
         <v>0.0630311205151477</v>
       </c>
       <c r="AW13" t="n">
-        <v>-0.4518192557963938</v>
+        <v>-0.4518192966162832</v>
       </c>
       <c r="AX13" t="n">
         <v>-0.2721097031519545</v>
       </c>
       <c r="AY13" t="n">
-        <v>0.2713425814751693</v>
+        <v>0.2713426912542354</v>
       </c>
       <c r="AZ13" t="inlineStr"/>
       <c r="BA13" t="n">
@@ -3940,16 +3940,16 @@
         <v>405.9760382080078</v>
       </c>
       <c r="AG18" t="n">
-        <v>361.2549255371094</v>
+        <v>361.2549249267578</v>
       </c>
       <c r="AH18" t="n">
         <v>-0.0147940676839341</v>
       </c>
       <c r="AI18" t="n">
-        <v>0.1071682984696545</v>
+        <v>0.1071683003402502</v>
       </c>
       <c r="AJ18" t="n">
-        <v>0.1237937797094604</v>
+        <v>0.1237937816081454</v>
       </c>
       <c r="AK18" t="n">
         <v>480.8090515136719</v>
@@ -3988,13 +3988,13 @@
         <v>0.4629652450487607</v>
       </c>
       <c r="AW18" t="n">
-        <v>8.384254085964638</v>
+        <v>8.384254925873597</v>
       </c>
       <c r="AX18" t="n">
         <v>0.154834014083173</v>
       </c>
       <c r="AY18" t="n">
-        <v>351.2130314740801</v>
+        <v>351.2129575265922</v>
       </c>
       <c r="AZ18" t="inlineStr"/>
       <c r="BA18" t="n">
@@ -4328,16 +4328,16 @@
         <v>261.3985458374024</v>
       </c>
       <c r="AG20" t="n">
-        <v>272.4722570037842</v>
+        <v>272.4722551727295</v>
       </c>
       <c r="AH20" t="n">
         <v>0.1000826214904216</v>
       </c>
       <c r="AI20" t="n">
-        <v>0.05537349277581693</v>
+        <v>0.05537349986808615</v>
       </c>
       <c r="AJ20" t="n">
-        <v>-0.0406416098583865</v>
+        <v>-0.04064160341135326</v>
       </c>
       <c r="AK20" t="n">
         <v>329.2300109863281</v>
@@ -4376,13 +4376,13 @@
         <v>0.02604071728593249</v>
       </c>
       <c r="AW20" t="n">
-        <v>1.612317035541202</v>
+        <v>1.612317397653624</v>
       </c>
       <c r="AX20" t="n">
-        <v>-0.000590030322446311</v>
+        <v>-0.0005899243216824779</v>
       </c>
       <c r="AY20" t="n">
-        <v>198.039346077303</v>
+        <v>198.0394610402244</v>
       </c>
       <c r="AZ20" t="inlineStr"/>
       <c r="BA20" t="n">
@@ -5102,16 +5102,16 @@
         <v>297.7269622802734</v>
       </c>
       <c r="AG24" t="n">
-        <v>272.096633682251</v>
+        <v>272.0966347503662</v>
       </c>
       <c r="AH24" t="n">
         <v>0.05909120527479672</v>
       </c>
       <c r="AI24" t="n">
-        <v>0.1588530260629508</v>
+        <v>0.1588530215138737</v>
       </c>
       <c r="AJ24" t="n">
-        <v>0.09419568427279046</v>
+        <v>0.09419567997752587</v>
       </c>
       <c r="AK24" t="n">
         <v>316.2200012207031</v>
@@ -5147,16 +5147,16 @@
         <v>0.2195252819657805</v>
       </c>
       <c r="AV24" t="n">
-        <v>0.4903770100349119</v>
+        <v>0.4903769025467106</v>
       </c>
       <c r="AW24" t="n">
         <v>1.311284607230153</v>
       </c>
       <c r="AX24" t="n">
-        <v>0.1656612312269863</v>
+        <v>0.1656610997217054</v>
       </c>
       <c r="AY24" t="n">
-        <v>3209.76902154225</v>
+        <v>3209.76780360039</v>
       </c>
       <c r="AZ24" t="inlineStr"/>
       <c r="BA24" t="n">
@@ -5659,10 +5659,10 @@
         </is>
       </c>
       <c r="Z27" t="n">
-        <v>0.1476428806781769</v>
+        <v>0.1477825343608856</v>
       </c>
       <c r="AA27" t="n">
-        <v>129868178973.3945</v>
+        <v>129991019772.6055</v>
       </c>
       <c r="AB27" t="inlineStr">
         <is>
@@ -6126,7 +6126,7 @@
         <v>1.789232944608137</v>
       </c>
       <c r="AY29" t="n">
-        <v>604.1799780628296</v>
+        <v>604.1797793213337</v>
       </c>
       <c r="AZ29" t="inlineStr"/>
       <c r="BA29" t="n">
@@ -6268,28 +6268,28 @@
         <v>209.0737417602539</v>
       </c>
       <c r="AG30" t="n">
-        <v>191.468422164917</v>
+        <v>191.468422088623</v>
       </c>
       <c r="AH30" t="n">
         <v>0.009022007918030539</v>
       </c>
       <c r="AI30" t="n">
-        <v>0.1018005179577943</v>
+        <v>0.1018005183968262</v>
       </c>
       <c r="AJ30" t="n">
-        <v>0.09194894592160452</v>
+        <v>0.09194894635671091</v>
       </c>
       <c r="AK30" t="n">
         <v>235.465576171875</v>
       </c>
       <c r="AL30" t="n">
-        <v>163.8517608642578</v>
+        <v>163.8517761230469</v>
       </c>
       <c r="AM30" t="n">
         <v>-0.1040728324556465</v>
       </c>
       <c r="AN30" t="n">
-        <v>0.287505276727761</v>
+        <v>0.287505156828106</v>
       </c>
       <c r="AO30" t="n">
         <v>50.27114310993102</v>
@@ -6316,7 +6316,7 @@
         <v>0.2872698368449687</v>
       </c>
       <c r="AW30" t="n">
-        <v>9.33287917561031</v>
+        <v>9.332877244964671</v>
       </c>
       <c r="AX30" t="n">
         <v>0.1184395258885382</v>
@@ -6509,16 +6509,16 @@
         <v>0.05062759896381297</v>
       </c>
       <c r="AV31" t="n">
-        <v>0.2140734622373373</v>
+        <v>0.2140733433376683</v>
       </c>
       <c r="AW31" t="n">
-        <v>0.477916035136061</v>
+        <v>0.4779155946520415</v>
       </c>
       <c r="AX31" t="n">
         <v>0.1046227422659505</v>
       </c>
       <c r="AY31" t="n">
-        <v>559.668694222702</v>
+        <v>559.668793274755</v>
       </c>
       <c r="AZ31" t="inlineStr"/>
       <c r="BA31" t="n">
@@ -6714,7 +6714,7 @@
         <v>1.555702248539101</v>
       </c>
       <c r="AY32" t="n">
-        <v>40.53741713740772</v>
+        <v>40.53742678010032</v>
       </c>
       <c r="AZ32" t="inlineStr"/>
       <c r="BA32" t="n">
@@ -6906,7 +6906,7 @@
         <v>3.003615150538764</v>
       </c>
       <c r="AY33" t="n">
-        <v>119.200901666593</v>
+        <v>119.2009174139452</v>
       </c>
       <c r="AZ33" t="inlineStr"/>
       <c r="BA33" t="n">
@@ -7098,7 +7098,7 @@
         <v>4.104878002897078</v>
       </c>
       <c r="AY34" t="n">
-        <v>33.78927898932974</v>
+        <v>33.78928770047334</v>
       </c>
       <c r="AZ34" t="inlineStr"/>
       <c r="BA34" t="n">
@@ -7290,7 +7290,7 @@
         <v>1.841141636730317</v>
       </c>
       <c r="AY35" t="n">
-        <v>28.33033194284154</v>
+        <v>28.33032159671425</v>
       </c>
       <c r="AZ35" t="inlineStr"/>
       <c r="BA35" t="n">
@@ -7482,7 +7482,7 @@
         <v>0.1234972253384632</v>
       </c>
       <c r="AY36" t="n">
-        <v>3.458769927801079</v>
+        <v>3.458769461191894</v>
       </c>
       <c r="AZ36" t="inlineStr"/>
       <c r="BA36" t="n">
@@ -7624,28 +7624,28 @@
         <v>74.7279963684082</v>
       </c>
       <c r="AG37" t="n">
-        <v>51.32824649810791</v>
+        <v>51.32824646949768</v>
       </c>
       <c r="AH37" t="n">
         <v>-0.05697991856643936</v>
       </c>
       <c r="AI37" t="n">
-        <v>0.3729282807917631</v>
+        <v>0.3729282815570296</v>
       </c>
       <c r="AJ37" t="n">
-        <v>0.4558844586900677</v>
+        <v>0.4558844595015739</v>
       </c>
       <c r="AK37" t="n">
         <v>93.55000305175781</v>
       </c>
       <c r="AL37" t="n">
-        <v>20.95925903320312</v>
+        <v>20.95926094055176</v>
       </c>
       <c r="AM37" t="n">
         <v>-0.2467129992319227</v>
       </c>
       <c r="AN37" t="n">
-        <v>2.362237238876925</v>
+        <v>2.362236932904371</v>
       </c>
       <c r="AO37" t="n">
         <v>33.62281192475615</v>
@@ -7669,16 +7669,16 @@
         <v>0.3859702206736597</v>
       </c>
       <c r="AV37" t="n">
-        <v>2.247039273833214</v>
+        <v>2.247039559198358</v>
       </c>
       <c r="AW37" t="n">
-        <v>2.26196568111741</v>
+        <v>2.261965393122681</v>
       </c>
       <c r="AX37" t="n">
         <v>0.6468892082431434</v>
       </c>
       <c r="AY37" t="n">
-        <v>4.697598058658468</v>
+        <v>4.697597619340071</v>
       </c>
       <c r="AZ37" t="inlineStr"/>
       <c r="BA37" t="n">
@@ -7810,22 +7810,22 @@
         <v>18.7</v>
       </c>
       <c r="AE38" t="n">
-        <v>191.8000030517578</v>
+        <v>186.8000030517578</v>
       </c>
       <c r="AF38" t="n">
-        <v>153.6120002746582</v>
+        <v>155.4720002746582</v>
       </c>
       <c r="AG38" t="n">
-        <v>69.94800010681152</v>
+        <v>70.77200012207031</v>
       </c>
       <c r="AH38" t="n">
-        <v>0.2486003873969447</v>
+        <v>0.2015025388607292</v>
       </c>
       <c r="AI38" t="n">
-        <v>1.742036981169965</v>
+        <v>1.639461972666561</v>
       </c>
       <c r="AJ38" t="n">
-        <v>1.196088523475877</v>
+        <v>1.196800994835444</v>
       </c>
       <c r="AK38" t="n">
         <v>239</v>
@@ -7834,13 +7834,13 @@
         <v>17.63999938964844</v>
       </c>
       <c r="AM38" t="n">
-        <v>-0.1974895269800928</v>
+        <v>-0.218410029072143</v>
       </c>
       <c r="AN38" t="n">
-        <v>9.873016422229046</v>
+        <v>9.589569700403528</v>
       </c>
       <c r="AO38" t="n">
-        <v>39.44444439211662</v>
+        <v>33.05194736351383</v>
       </c>
       <c r="AP38" t="n">
         <v>77156</v>
@@ -7852,25 +7852,25 @@
         <v>0.4156891234118705</v>
       </c>
       <c r="AS38" t="n">
-        <v>0.341258762599705</v>
+        <v>0.2114137921446129</v>
       </c>
       <c r="AT38" t="n">
-        <v>1.89291092342827</v>
+        <v>1.703328613266424</v>
       </c>
       <c r="AU38" t="n">
-        <v>4.616398081458695</v>
+        <v>4.461988271479282</v>
       </c>
       <c r="AV38" t="n">
-        <v>8.775738779186103</v>
+        <v>8.434343951999546</v>
       </c>
       <c r="AW38" t="n">
-        <v>4.263584246605888</v>
+        <v>4.169031013974967</v>
       </c>
       <c r="AX38" t="n">
-        <v>4.847561204667469</v>
+        <v>4.69512217673144</v>
       </c>
       <c r="AY38" t="n">
-        <v>15.71474529855174</v>
+        <v>15.27901294365783</v>
       </c>
       <c r="AZ38" t="inlineStr"/>
       <c r="BA38" t="n">
@@ -8012,16 +8012,16 @@
         <v>125.4860302734375</v>
       </c>
       <c r="AG39" t="n">
-        <v>104.0938962936401</v>
+        <v>104.0938962173462</v>
       </c>
       <c r="AH39" t="n">
         <v>-0.03168502604268508</v>
       </c>
       <c r="AI39" t="n">
-        <v>0.1673114991628419</v>
+        <v>0.1673115000184042</v>
       </c>
       <c r="AJ39" t="n">
-        <v>0.205508053223908</v>
+        <v>0.2055080541074659</v>
       </c>
       <c r="AK39" t="n">
         <v>133.0599975585938</v>
@@ -8057,16 +8057,16 @@
         <v>0.4124845916784821</v>
       </c>
       <c r="AV39" t="n">
-        <v>0.2697068511936827</v>
+        <v>0.2697067499693466</v>
       </c>
       <c r="AW39" t="n">
-        <v>2.452222075910021</v>
+        <v>2.452222450059847</v>
       </c>
       <c r="AX39" t="n">
         <v>0.4817174890207807</v>
       </c>
       <c r="AY39" t="n">
-        <v>104.4620601888137</v>
+        <v>104.4620383655108</v>
       </c>
       <c r="AZ39" t="inlineStr"/>
       <c r="BA39" t="n">
@@ -8204,16 +8204,16 @@
         <v>2684.7</v>
       </c>
       <c r="AG40" t="n">
-        <v>2602.836932373047</v>
+        <v>2602.83692993164</v>
       </c>
       <c r="AH40" t="n">
         <v>0.03940850001862417</v>
       </c>
       <c r="AI40" t="n">
-        <v>0.07209943323489654</v>
+        <v>0.07209943424050325</v>
       </c>
       <c r="AJ40" t="n">
-        <v>0.03145147765838607</v>
+        <v>0.03145147862586595</v>
       </c>
       <c r="AK40" t="n">
         <v>2808</v>
@@ -8249,7 +8249,7 @@
         <v>0.03854153539012617</v>
       </c>
       <c r="AV40" t="n">
-        <v>0.160986175495293</v>
+        <v>0.1609860575686113</v>
       </c>
       <c r="AW40" t="n">
         <v>0.7531327201194351</v>
@@ -8258,7 +8258,7 @@
         <v>0.03607197425947772</v>
       </c>
       <c r="AY40" t="n">
-        <v>3.264597949503009</v>
+        <v>3.264597551712717</v>
       </c>
       <c r="AZ40" t="inlineStr"/>
       <c r="BA40" t="n">
@@ -8400,16 +8400,16 @@
         <v>1066.220737304687</v>
       </c>
       <c r="AG41" t="n">
-        <v>906.3318444824218</v>
+        <v>906.3318453979492</v>
       </c>
       <c r="AH41" t="n">
         <v>-0.01407848847991211</v>
       </c>
       <c r="AI41" t="n">
-        <v>0.1598510714779238</v>
+        <v>0.159851070306305</v>
       </c>
       <c r="AJ41" t="n">
-        <v>0.1764131910355342</v>
+        <v>0.1764131898471852</v>
       </c>
       <c r="AK41" t="n">
         <v>1115.93994140625</v>
@@ -8454,7 +8454,7 @@
         <v>0.3900707617105812</v>
       </c>
       <c r="AY41" t="n">
-        <v>2.403099240424091</v>
+        <v>2.403098904214745</v>
       </c>
       <c r="AZ41" t="inlineStr"/>
       <c r="BA41" t="n">
@@ -8836,13 +8836,13 @@
         <v>0.08879809751909096</v>
       </c>
       <c r="AW43" t="n">
-        <v>0.424025524989234</v>
+        <v>0.424025782257571</v>
       </c>
       <c r="AX43" t="n">
         <v>0.1794454765270563</v>
       </c>
       <c r="AY43" t="n">
-        <v>34.3910593674331</v>
+        <v>34.39106598848021</v>
       </c>
       <c r="AZ43" t="inlineStr"/>
       <c r="BA43" t="n">
@@ -9034,7 +9034,7 @@
         <v>0.02366607311174418</v>
       </c>
       <c r="AY44" t="n">
-        <v>3.011992539465282</v>
+        <v>3.011993824378248</v>
       </c>
       <c r="AZ44" t="inlineStr"/>
       <c r="BA44" t="n">
@@ -9416,7 +9416,7 @@
         <v>-0.05892355276542649</v>
       </c>
       <c r="AY46" t="n">
-        <v>0.6047316879760181</v>
+        <v>0.6047306231019427</v>
       </c>
       <c r="AZ46" t="inlineStr"/>
       <c r="BA46" t="n">
@@ -9912,28 +9912,28 @@
         <v>66.27910278320313</v>
       </c>
       <c r="AG49" t="n">
-        <v>61.4878981590271</v>
+        <v>61.48789806365967</v>
       </c>
       <c r="AH49" t="n">
         <v>0.05734686934861166</v>
       </c>
       <c r="AI49" t="n">
-        <v>0.1397364998524702</v>
+        <v>0.1397365016201959</v>
       </c>
       <c r="AJ49" t="n">
-        <v>0.07792109939722547</v>
+        <v>0.0779211010690759</v>
       </c>
       <c r="AK49" t="n">
         <v>70.08000183105469</v>
       </c>
       <c r="AL49" t="n">
-        <v>54.15811157226562</v>
+        <v>54.15811538696289</v>
       </c>
       <c r="AM49" t="n">
         <v>0</v>
       </c>
       <c r="AN49" t="n">
-        <v>0.2939890220792458</v>
+        <v>0.2939889309354469</v>
       </c>
       <c r="AO49" t="n">
         <v>60.91500764933151</v>
@@ -9960,13 +9960,13 @@
         <v>0.2581684321906936</v>
       </c>
       <c r="AW49" t="n">
-        <v>0.1802576874737116</v>
+        <v>0.1802579907788389</v>
       </c>
       <c r="AX49" t="n">
         <v>0.207563158772776</v>
       </c>
       <c r="AY49" t="n">
-        <v>188.63773634206</v>
+        <v>188.6378433962856</v>
       </c>
       <c r="AZ49" t="inlineStr"/>
       <c r="BA49" t="n">
@@ -10160,7 +10160,7 @@
         <v>0.6092896408427024</v>
       </c>
       <c r="AY50" t="n">
-        <v>7.351867541581512</v>
+        <v>7.351868516651404</v>
       </c>
       <c r="AZ50" t="inlineStr"/>
       <c r="BA50" t="n">
@@ -10302,16 +10302,16 @@
         <v>14.5815599822998</v>
       </c>
       <c r="AG51" t="n">
-        <v>14.23315340995789</v>
+        <v>14.23315336227417</v>
       </c>
       <c r="AH51" t="n">
         <v>0.01360895205398238</v>
       </c>
       <c r="AI51" t="n">
-        <v>0.03842060204527242</v>
+        <v>0.03842060552417514</v>
       </c>
       <c r="AJ51" t="n">
-        <v>0.02447852294616348</v>
+        <v>0.02447852637835735</v>
       </c>
       <c r="AK51" t="n">
         <v>17.06953239440918</v>
@@ -10344,19 +10344,19 @@
         <v>0.03976638797694187</v>
       </c>
       <c r="AU51" t="n">
-        <v>0.06465544779208687</v>
+        <v>0.06465552093021687</v>
       </c>
       <c r="AV51" t="n">
         <v>0.2522044132542418</v>
       </c>
       <c r="AW51" t="n">
-        <v>-0.3125524802434755</v>
+        <v>-0.3125526022167473</v>
       </c>
       <c r="AX51" t="n">
         <v>0.02155212588028221</v>
       </c>
       <c r="AY51" t="n">
-        <v>6.406423842467975</v>
+        <v>6.406424284906384</v>
       </c>
       <c r="AZ51" t="inlineStr"/>
       <c r="BA51" t="n">
@@ -10688,16 +10688,16 @@
         <v>124.7692489624023</v>
       </c>
       <c r="AG53" t="n">
-        <v>122.871420249939</v>
+        <v>122.8714202880859</v>
       </c>
       <c r="AH53" t="n">
         <v>0.005696551036749709</v>
       </c>
       <c r="AI53" t="n">
-        <v>0.02123018600817317</v>
+        <v>0.02123018569111945</v>
       </c>
       <c r="AJ53" t="n">
-        <v>0.0154456480490166</v>
+        <v>0.01544564773375878</v>
       </c>
       <c r="AK53" t="n">
         <v>132.3166198730469</v>
@@ -10733,7 +10733,7 @@
         <v>0.08798379294662428</v>
       </c>
       <c r="AV53" t="n">
-        <v>0.09896576276649749</v>
+        <v>0.09896568933475258</v>
       </c>
       <c r="AW53" t="n">
         <v>0.529614046443887</v>
@@ -10742,7 +10742,7 @@
         <v>0.08687203524002696</v>
       </c>
       <c r="AY53" t="n">
-        <v>168.4898088985315</v>
+        <v>168.4896724426017</v>
       </c>
       <c r="AZ53" t="inlineStr"/>
       <c r="BA53" t="n">
@@ -10929,16 +10929,16 @@
         <v>0.2768792389174044</v>
       </c>
       <c r="AV54" t="n">
-        <v>0.4368560101023142</v>
+        <v>0.4368558731939771</v>
       </c>
       <c r="AW54" t="n">
-        <v>1.699661016949153</v>
+        <v>1.699660533643547</v>
       </c>
       <c r="AX54" t="n">
         <v>0.2405563051351287</v>
       </c>
       <c r="AY54" t="n">
-        <v>213.0600145167256</v>
+        <v>213.0600382558457</v>
       </c>
       <c r="AZ54" t="inlineStr"/>
       <c r="BA54" t="n">
@@ -11080,28 +11080,28 @@
         <v>45.56361747741699</v>
       </c>
       <c r="AG55" t="n">
-        <v>45.45492044448852</v>
+        <v>45.45492042541504</v>
       </c>
       <c r="AH55" t="n">
         <v>0.02713528530205833</v>
       </c>
       <c r="AI55" t="n">
-        <v>0.02959148931334488</v>
+        <v>0.02959148974537507</v>
       </c>
       <c r="AJ55" t="n">
-        <v>0.002391314996606608</v>
+        <v>0.002391315417223261</v>
       </c>
       <c r="AK55" t="n">
         <v>49.82146072387695</v>
       </c>
       <c r="AL55" t="n">
-        <v>41.35774993896484</v>
+        <v>41.35775375366211</v>
       </c>
       <c r="AM55" t="n">
         <v>-0.06064578281961874</v>
       </c>
       <c r="AN55" t="n">
-        <v>0.1315895885566138</v>
+        <v>0.1315894841826737</v>
       </c>
       <c r="AO55" t="n">
         <v>56.50457813303605</v>
@@ -11125,16 +11125,16 @@
         <v>0.09653907045408494</v>
       </c>
       <c r="AV55" t="n">
-        <v>0.1113595325389343</v>
+        <v>0.1113594318635374</v>
       </c>
       <c r="AW55" t="n">
-        <v>0.7342669768602337</v>
+        <v>0.7342668542812223</v>
       </c>
       <c r="AX55" t="n">
         <v>0.08480475291928924</v>
       </c>
       <c r="AY55" t="n">
-        <v>189.8671427079904</v>
+        <v>189.8669339184967</v>
       </c>
       <c r="AZ55" t="inlineStr"/>
       <c r="BA55" t="n">
@@ -11276,16 +11276,16 @@
         <v>88.69704376220703</v>
       </c>
       <c r="AG56" t="n">
-        <v>85.99043495178222</v>
+        <v>85.99043476104737</v>
       </c>
       <c r="AH56" t="n">
         <v>-0.008309687070409688</v>
       </c>
       <c r="AI56" t="n">
-        <v>0.02290445598739943</v>
+        <v>0.02290445825629761</v>
       </c>
       <c r="AJ56" t="n">
-        <v>0.03147569624391955</v>
+        <v>0.03147569853182941</v>
       </c>
       <c r="AK56" t="n">
         <v>97.16828918457031</v>
@@ -11321,7 +11321,7 @@
         <v>0.1222597138586909</v>
       </c>
       <c r="AV56" t="n">
-        <v>0.212580508059667</v>
+        <v>0.2125803805256681</v>
       </c>
       <c r="AW56" t="n">
         <v>0.3505196278270164</v>
@@ -11330,7 +11330,7 @@
         <v>0.1022911005985252</v>
       </c>
       <c r="AY56" t="n">
-        <v>252.1195017895775</v>
+        <v>252.1195669130385</v>
       </c>
       <c r="AZ56" t="inlineStr"/>
       <c r="BA56" t="n">
@@ -11472,28 +11472,28 @@
         <v>93.83682312011719</v>
       </c>
       <c r="AG57" t="n">
-        <v>91.68827781677246</v>
+        <v>91.68827754974365</v>
       </c>
       <c r="AH57" t="n">
         <v>0.01889639302861523</v>
       </c>
       <c r="AI57" t="n">
-        <v>0.04277234655248052</v>
+        <v>0.04277234958940368</v>
       </c>
       <c r="AJ57" t="n">
-        <v>0.02343315148353353</v>
+        <v>0.02343315446413419</v>
       </c>
       <c r="AK57" t="n">
         <v>98.29612731933594</v>
       </c>
       <c r="AL57" t="n">
-        <v>82.73965454101562</v>
+        <v>82.73964691162109</v>
       </c>
       <c r="AM57" t="n">
         <v>-0.02732688237307579</v>
       </c>
       <c r="AN57" t="n">
-        <v>0.1555523302669322</v>
+        <v>0.1555524368200172</v>
       </c>
       <c r="AO57" t="n">
         <v>58.50202575045431</v>
@@ -11514,10 +11514,10 @@
         <v>-0.007703253736871862</v>
       </c>
       <c r="AU57" t="n">
-        <v>0.1139515030236831</v>
+        <v>0.1139514040045131</v>
       </c>
       <c r="AV57" t="n">
-        <v>0.05870520556638703</v>
+        <v>0.05870511612535267</v>
       </c>
       <c r="AW57" t="n">
         <v>0.8689427817012998</v>
@@ -11526,7 +11526,7 @@
         <v>0.1144625773375663</v>
       </c>
       <c r="AY57" t="n">
-        <v>351.5557162207932</v>
+        <v>351.5555999894062</v>
       </c>
       <c r="AZ57" t="inlineStr"/>
       <c r="BA57" t="n">
@@ -11658,22 +11658,22 @@
         <v>5.8</v>
       </c>
       <c r="AE58" t="n">
-        <v>156.2400054931641</v>
+        <v>152.1199951171875</v>
       </c>
       <c r="AF58" t="n">
-        <v>166.0171997070312</v>
+        <v>165.4479995727539</v>
       </c>
       <c r="AG58" t="n">
-        <v>140.8513035583496</v>
+        <v>141.1316515350342</v>
       </c>
       <c r="AH58" t="n">
-        <v>-0.05889265829757928</v>
+        <v>-0.08055706016382236</v>
       </c>
       <c r="AI58" t="n">
-        <v>0.109254948630557</v>
+        <v>0.07785881807969641</v>
       </c>
       <c r="AJ58" t="n">
-        <v>0.1786699555695366</v>
+        <v>0.1722954969579131</v>
       </c>
       <c r="AK58" t="n">
         <v>187.6199951171875</v>
@@ -11682,43 +11682,43 @@
         <v>84.04161071777344</v>
       </c>
       <c r="AM58" t="n">
-        <v>-0.1672529071564227</v>
+        <v>-0.1892122424255831</v>
       </c>
       <c r="AN58" t="n">
-        <v>0.8590791413773062</v>
+        <v>0.8100556833451622</v>
       </c>
       <c r="AO58" t="n">
-        <v>40.53167358431317</v>
+        <v>37.99041104592384</v>
       </c>
       <c r="AP58" t="n">
-        <v>1526536</v>
+        <v>1528158</v>
       </c>
       <c r="AQ58" t="n">
-        <v>2545502.56</v>
+        <v>2545535</v>
       </c>
       <c r="AR58" t="n">
-        <v>0.5996992593871129</v>
+        <v>0.6003288110357941</v>
       </c>
       <c r="AS58" t="n">
-        <v>0.06285718022560594</v>
+        <v>-0.009506489754266712</v>
       </c>
       <c r="AT58" t="n">
-        <v>-0.05822778034185938</v>
+        <v>-0.1102012801637982</v>
       </c>
       <c r="AU58" t="n">
-        <v>0.223917913841903</v>
+        <v>0.1719883418775445</v>
       </c>
       <c r="AV58" t="n">
-        <v>0.7114558292045023</v>
+        <v>0.6598076692550514</v>
       </c>
       <c r="AW58" t="n">
-        <v>5.875139167106532</v>
+        <v>5.590419621851969</v>
       </c>
       <c r="AX58" t="n">
-        <v>0.2777383831769491</v>
+        <v>0.2440447374307393</v>
       </c>
       <c r="AY58" t="n">
-        <v>6.16889543551419</v>
+        <v>5.97985282171642</v>
       </c>
       <c r="AZ58" t="inlineStr"/>
       <c r="BA58" t="n">
@@ -11858,16 +11858,16 @@
         <v>153.8592938232422</v>
       </c>
       <c r="AG59" t="n">
-        <v>166.7918190765381</v>
+        <v>166.7918186187744</v>
       </c>
       <c r="AH59" t="n">
         <v>0.03250181814076392</v>
       </c>
       <c r="AI59" t="n">
-        <v>-0.04755520090914489</v>
+        <v>-0.0475551982951401</v>
       </c>
       <c r="AJ59" t="n">
-        <v>-0.07753692791947642</v>
+        <v>-0.07753692538775714</v>
       </c>
       <c r="AK59" t="n">
         <v>217.0162200927734</v>
@@ -11903,16 +11903,16 @@
         <v>0.05776533874442791</v>
       </c>
       <c r="AV59" t="n">
-        <v>-0.1843226309643335</v>
+        <v>-0.1843225670582255</v>
       </c>
       <c r="AW59" t="n">
-        <v>8.152996012891588</v>
+        <v>8.152997018762193</v>
       </c>
       <c r="AX59" t="n">
-        <v>-0.03589257536134183</v>
+        <v>-0.0358924860808848</v>
       </c>
       <c r="AY59" t="n">
-        <v>13.01174408365016</v>
+        <v>13.01174290504081</v>
       </c>
       <c r="AZ59" t="inlineStr"/>
       <c r="BA59" t="n">
@@ -12065,13 +12065,13 @@
         <v>238.1012115478516</v>
       </c>
       <c r="AL60" t="n">
-        <v>135.6905517578125</v>
+        <v>135.6905670166016</v>
       </c>
       <c r="AM60" t="n">
         <v>-0.2188195986452622</v>
       </c>
       <c r="AN60" t="n">
-        <v>0.3707660378003503</v>
+        <v>0.3707658836538221</v>
       </c>
       <c r="AO60" t="n">
         <v>32.9285538579864</v>
@@ -12095,7 +12095,7 @@
         <v>-0.03464766810121545</v>
       </c>
       <c r="AV60" t="n">
-        <v>0.3707660378003503</v>
+        <v>0.3707658836538221</v>
       </c>
       <c r="AW60" t="n">
         <v>2.365315022323721</v>
@@ -12104,7 +12104,7 @@
         <v>0.02560388456948459</v>
       </c>
       <c r="AY60" t="n">
-        <v>12.12652192269306</v>
+        <v>12.12652368961162</v>
       </c>
       <c r="AZ60" t="inlineStr"/>
       <c r="BA60" t="n">
@@ -12290,13 +12290,13 @@
         <v>0.3580471866742656</v>
       </c>
       <c r="AW61" t="n">
-        <v>4.074691322172047</v>
+        <v>4.074690810462737</v>
       </c>
       <c r="AX61" t="n">
         <v>-0.02607548456255149</v>
       </c>
       <c r="AY61" t="n">
-        <v>15.04248294368242</v>
+        <v>15.04247782984243</v>
       </c>
       <c r="AZ61" t="inlineStr"/>
       <c r="BA61" t="n">
@@ -12630,25 +12630,25 @@
         <v>273.078256225586</v>
       </c>
       <c r="AG63" t="n">
-        <v>314.0618740844727</v>
+        <v>314.0618737792969</v>
       </c>
       <c r="AH63" t="n">
         <v>-0.07945799728869241</v>
       </c>
       <c r="AI63" t="n">
-        <v>-0.1995844589044283</v>
+        <v>-0.1995844581266598</v>
       </c>
       <c r="AJ63" t="n">
-        <v>-0.130495361712907</v>
+        <v>-0.1304953608680042</v>
       </c>
       <c r="AK63" t="n">
-        <v>402.3219299316406</v>
+        <v>402.3219604492188</v>
       </c>
       <c r="AL63" t="n">
         <v>236.5</v>
       </c>
       <c r="AM63" t="n">
-        <v>-0.3751769759964986</v>
+        <v>-0.3751770233915884</v>
       </c>
       <c r="AN63" t="n">
         <v>0.06291756821485195</v>
@@ -12874,7 +12874,7 @@
         <v>-0.3722935667825401</v>
       </c>
       <c r="AY64" t="n">
-        <v>-0.9213619079351065</v>
+        <v>-0.9213619167614913</v>
       </c>
       <c r="AZ64" t="inlineStr"/>
       <c r="BA64" t="n">
@@ -13016,16 +13016,16 @@
         <v>137.554800567627</v>
       </c>
       <c r="AG65" t="n">
-        <v>154.7436396408081</v>
+        <v>154.7436395645142</v>
       </c>
       <c r="AH65" t="n">
         <v>0.02082949914866639</v>
       </c>
       <c r="AI65" t="n">
-        <v>-0.09256368471822762</v>
+        <v>-0.09256368427083028</v>
       </c>
       <c r="AJ65" t="n">
-        <v>-0.1110794544646875</v>
+        <v>-0.1110794540264189</v>
       </c>
       <c r="AK65" t="n">
         <v>183.4681396484375</v>
@@ -13061,7 +13061,7 @@
         <v>-0.01560841976449645</v>
       </c>
       <c r="AV65" t="n">
-        <v>-0.06166660089967213</v>
+        <v>-0.06166669657620116</v>
       </c>
       <c r="AW65" t="n">
         <v>2.883612305762729</v>
@@ -13070,7 +13070,7 @@
         <v>-0.1496766437851758</v>
       </c>
       <c r="AY65" t="n">
-        <v>18.60044344292323</v>
+        <v>18.60044083375033</v>
       </c>
       <c r="AZ65" t="inlineStr"/>
       <c r="BA65" t="n">
@@ -13594,16 +13594,16 @@
         <v>145.2885821533203</v>
       </c>
       <c r="AG68" t="n">
-        <v>116.4364813995361</v>
+        <v>116.4364813613892</v>
       </c>
       <c r="AH68" t="n">
         <v>0.1623074065034387</v>
       </c>
       <c r="AI68" t="n">
-        <v>0.4503186036490816</v>
+        <v>0.4503186041242357</v>
       </c>
       <c r="AJ68" t="n">
-        <v>0.2477926196926379</v>
+        <v>0.2477926201014404</v>
       </c>
       <c r="AK68" t="n">
         <v>180.5316925048828</v>
@@ -13639,16 +13639,16 @@
         <v>0.6129842513774852</v>
       </c>
       <c r="AV68" t="n">
-        <v>0.6145965570791305</v>
+        <v>0.6145964393007453</v>
       </c>
       <c r="AW68" t="n">
-        <v>1.293937816756738</v>
+        <v>1.293938292235311</v>
       </c>
       <c r="AX68" t="n">
         <v>0.5990466171336413</v>
       </c>
       <c r="AY68" t="n">
-        <v>179.0869021166676</v>
+        <v>179.0868906696635</v>
       </c>
       <c r="AZ68" t="inlineStr"/>
       <c r="BA68" t="n">
@@ -13949,10 +13949,10 @@
         </is>
       </c>
       <c r="Z70" t="n">
-        <v>0.0006672449526377022</v>
+        <v>0.0006671692826785147</v>
       </c>
       <c r="AA70" t="n">
-        <v>1032550685492.281</v>
+        <v>1032433587464.156</v>
       </c>
       <c r="AB70" t="inlineStr">
         <is>
@@ -14017,16 +14017,16 @@
         <v>2.008798838852081</v>
       </c>
       <c r="AV70" t="n">
-        <v>6.496951139566664</v>
+        <v>6.496950333886184</v>
       </c>
       <c r="AW70" t="n">
-        <v>18.40183875253074</v>
+        <v>18.4018414505769</v>
       </c>
       <c r="AX70" t="n">
         <v>2.226570064441672</v>
       </c>
       <c r="AY70" t="n">
-        <v>-10.52489727727343</v>
+        <v>-10.52490182906515</v>
       </c>
       <c r="AZ70" t="inlineStr"/>
       <c r="BA70" t="n">
@@ -14145,10 +14145,10 @@
         </is>
       </c>
       <c r="Z71" t="n">
-        <v>0.0006672449526377022</v>
+        <v>0.0006671692826785147</v>
       </c>
       <c r="AA71" t="n">
-        <v>1248729263492.984</v>
+        <v>1248587649394.547</v>
       </c>
       <c r="AB71" t="inlineStr">
         <is>
@@ -14168,16 +14168,16 @@
         <v>303340</v>
       </c>
       <c r="AG71" t="n">
-        <v>181070.4312890625</v>
+        <v>181070.43125</v>
       </c>
       <c r="AH71" t="n">
         <v>-0.06046020966572163</v>
       </c>
       <c r="AI71" t="n">
-        <v>0.5739731659722145</v>
+        <v>0.5739731663117691</v>
       </c>
       <c r="AJ71" t="n">
-        <v>0.6752597198807422</v>
+        <v>0.6752597202421475</v>
       </c>
       <c r="AK71" t="n">
         <v>362500</v>
@@ -14408,13 +14408,13 @@
         <v>7.388845264110813</v>
       </c>
       <c r="AW72" t="n">
-        <v>5.28095282343382</v>
+        <v>5.280951970792506</v>
       </c>
       <c r="AX72" t="n">
         <v>0.9540096451224696</v>
       </c>
       <c r="AY72" t="n">
-        <v>3.636716879610193</v>
+        <v>3.636716414948917</v>
       </c>
       <c r="AZ72" t="inlineStr"/>
       <c r="BA72" t="n">
@@ -14600,13 +14600,13 @@
         <v>7.227866436434194</v>
       </c>
       <c r="AW73" t="n">
-        <v>4.912028806014082</v>
+        <v>4.912029418329285</v>
       </c>
       <c r="AX73" t="n">
         <v>1.11062651104741</v>
       </c>
       <c r="AY73" t="n">
-        <v>-0.4918197389740576</v>
+        <v>-0.4918198475537601</v>
       </c>
       <c r="AZ73" t="inlineStr"/>
       <c r="BA73" t="n">
@@ -14748,16 +14748,16 @@
         <v>329.1420672607422</v>
       </c>
       <c r="AG74" t="n">
-        <v>227.9347861862183</v>
+        <v>227.9347863006592</v>
       </c>
       <c r="AH74" t="n">
         <v>0.06437317322534364</v>
       </c>
       <c r="AI74" t="n">
-        <v>0.5369746427649391</v>
+        <v>0.5369746419932591</v>
       </c>
       <c r="AJ74" t="n">
-        <v>0.4440185842973505</v>
+        <v>0.4440185835723414</v>
       </c>
       <c r="AK74" t="n">
         <v>433.3299865722656</v>
@@ -14796,13 +14796,13 @@
         <v>2.485740056595084</v>
       </c>
       <c r="AW74" t="n">
-        <v>4.844537693193175</v>
+        <v>4.844538437090752</v>
       </c>
       <c r="AX74" t="n">
         <v>0.8966647974746411</v>
       </c>
       <c r="AY74" t="n">
-        <v>1857.200146520424</v>
+        <v>1857.199852784066</v>
       </c>
       <c r="AZ74" t="inlineStr"/>
       <c r="BA74" t="n">
@@ -14944,28 +14944,28 @@
         <v>898.9240441894531</v>
       </c>
       <c r="AG75" t="n">
-        <v>464.3001769256592</v>
+        <v>464.3001767730713</v>
       </c>
       <c r="AH75" t="n">
         <v>0.08941349841853374</v>
       </c>
       <c r="AI75" t="n">
-        <v>1.109195810084234</v>
+        <v>1.109195810777401</v>
       </c>
       <c r="AJ75" t="n">
-        <v>0.9360837855837887</v>
+        <v>0.9360837862200644</v>
       </c>
       <c r="AK75" t="n">
         <v>1213.373413085938</v>
       </c>
       <c r="AL75" t="n">
-        <v>104.7119369506836</v>
+        <v>104.7119293212891</v>
       </c>
       <c r="AM75" t="n">
         <v>-0.1929112858156803</v>
       </c>
       <c r="AN75" t="n">
-        <v>8.352324255583122</v>
+        <v>8.352324937000912</v>
       </c>
       <c r="AO75" t="n">
         <v>40.4435338385203</v>
@@ -14989,16 +14989,16 @@
         <v>1.996336946400833</v>
       </c>
       <c r="AV75" t="n">
-        <v>6.96744168695323</v>
+        <v>6.967442181505431</v>
       </c>
       <c r="AW75" t="n">
-        <v>11.50179167064778</v>
+        <v>11.50178801772941</v>
       </c>
       <c r="AX75" t="n">
-        <v>2.106530793808759</v>
+        <v>2.106531094544943</v>
       </c>
       <c r="AY75" t="n">
-        <v>724.0062980070579</v>
+        <v>724.0062340221026</v>
       </c>
       <c r="AZ75" t="inlineStr"/>
       <c r="BA75" t="n">
@@ -15530,28 +15530,28 @@
         <v>868.2855505371094</v>
       </c>
       <c r="AG78" t="n">
-        <v>472.2589469909668</v>
+        <v>472.2589468383789</v>
       </c>
       <c r="AH78" t="n">
         <v>0.04843392394626966</v>
       </c>
       <c r="AI78" t="n">
-        <v>0.9276289685050294</v>
+        <v>0.9276289691278508</v>
       </c>
       <c r="AJ78" t="n">
-        <v>0.8385793558162438</v>
+        <v>0.838579356410293</v>
       </c>
       <c r="AK78" t="n">
         <v>1093.260498046875</v>
       </c>
       <c r="AL78" t="n">
-        <v>143.3166656494141</v>
+        <v>143.316650390625</v>
       </c>
       <c r="AM78" t="n">
         <v>-0.1673164552439206</v>
       </c>
       <c r="AN78" t="n">
-        <v>5.351948133389961</v>
+        <v>5.351948809675908</v>
       </c>
       <c r="AO78" t="n">
         <v>38.12116368120392</v>
@@ -15575,16 +15575,16 @@
         <v>2.20799457899861</v>
       </c>
       <c r="AV78" t="n">
-        <v>5.351948133389961</v>
+        <v>5.351948809675908</v>
       </c>
       <c r="AW78" t="n">
-        <v>11.14208755627236</v>
+        <v>11.142091263033</v>
       </c>
       <c r="AX78" t="n">
         <v>2.173743552772943</v>
       </c>
       <c r="AY78" t="n">
-        <v>171.6941981062739</v>
+        <v>171.6942605921833</v>
       </c>
       <c r="AZ78" t="inlineStr"/>
       <c r="BA78" t="n">
@@ -15724,16 +15724,16 @@
         <v>546.2103399658204</v>
       </c>
       <c r="AG79" t="n">
-        <v>301.8788362121582</v>
+        <v>301.8788361740112</v>
       </c>
       <c r="AH79" t="n">
         <v>0.06660380484910799</v>
       </c>
       <c r="AI79" t="n">
-        <v>0.9298803260458737</v>
+        <v>0.9298803262897435</v>
       </c>
       <c r="AJ79" t="n">
-        <v>0.8093694371537454</v>
+        <v>0.8093694373823868</v>
       </c>
       <c r="AK79" t="n">
         <v>746.22998046875</v>
@@ -15778,7 +15778,7 @@
         <v>2.106131402193798</v>
       </c>
       <c r="AY79" t="n">
-        <v>856.330175539636</v>
+        <v>856.3301003404326</v>
       </c>
       <c r="AZ79" t="inlineStr"/>
       <c r="BA79" t="n">
@@ -16278,13 +16278,13 @@
         <v>0.6289717605625493</v>
       </c>
       <c r="AW82" t="n">
-        <v>3.757894722428535</v>
+        <v>3.757894179517444</v>
       </c>
       <c r="AX82" t="n">
         <v>0.1424722954066484</v>
       </c>
       <c r="AY82" t="n">
-        <v>1270.11682618042</v>
+        <v>1270.116977547045</v>
       </c>
       <c r="AZ82" t="inlineStr"/>
       <c r="BA82" t="n">
@@ -16399,10 +16399,10 @@
         </is>
       </c>
       <c r="Z83" t="n">
-        <v>0.1476428806781769</v>
+        <v>0.1477825343608856</v>
       </c>
       <c r="AA83" t="n">
-        <v>180130868353.9062</v>
+        <v>180301252046.0938</v>
       </c>
       <c r="AB83" t="inlineStr">
         <is>
@@ -16470,13 +16470,13 @@
         <v>6.921959468381198</v>
       </c>
       <c r="AW83" t="n">
-        <v>33.3001757526419</v>
+        <v>33.30017780386748</v>
       </c>
       <c r="AX83" t="n">
         <v>0.7566271538047729</v>
       </c>
       <c r="AY83" t="n">
-        <v>235.375636016669</v>
+        <v>235.3755873091461</v>
       </c>
       <c r="AZ83" t="inlineStr"/>
       <c r="BA83" t="n">
@@ -16608,22 +16608,22 @@
         <v>25.1</v>
       </c>
       <c r="AE84" t="n">
-        <v>132.8000030517578</v>
+        <v>134</v>
       </c>
       <c r="AF84" t="n">
-        <v>152.6272821044922</v>
+        <v>152.2020959472656</v>
       </c>
       <c r="AG84" t="n">
-        <v>130.9495380401611</v>
+        <v>130.9763069152832</v>
       </c>
       <c r="AH84" t="n">
-        <v>-0.129906519852461</v>
+        <v>-0.1195916247669297</v>
       </c>
       <c r="AI84" t="n">
-        <v>0.01413113050486015</v>
+        <v>0.02308580197388332</v>
       </c>
       <c r="AJ84" t="n">
-        <v>0.1655427303430628</v>
+        <v>0.1620582342859269</v>
       </c>
       <c r="AK84" t="n">
         <v>164.8832092285156</v>
@@ -16632,13 +16632,13 @@
         <v>108.1217498779297</v>
       </c>
       <c r="AM84" t="n">
-        <v>-0.1945814029631903</v>
+        <v>-0.1873035427501526</v>
       </c>
       <c r="AN84" t="n">
-        <v>0.2282450404445919</v>
+        <v>0.2393436117274004</v>
       </c>
       <c r="AO84" t="n">
-        <v>21.86146070926314</v>
+        <v>23.51693887882772</v>
       </c>
       <c r="AP84" t="n">
         <v>145970</v>
@@ -16650,25 +16650,25 @@
         <v>1.114166114176037</v>
       </c>
       <c r="AS84" t="n">
-        <v>-0.09413371403281867</v>
+        <v>-0.08156267576630183</v>
       </c>
       <c r="AT84" t="n">
-        <v>0.04343959838661671</v>
+        <v>0.02364382542268406</v>
       </c>
       <c r="AU84" t="n">
-        <v>0.09942912480414901</v>
+        <v>0.1013053149894143</v>
       </c>
       <c r="AV84" t="n">
-        <v>0.2020424490466763</v>
+        <v>0.2393436117274004</v>
       </c>
       <c r="AW84" t="n">
-        <v>0.8421877191097866</v>
+        <v>0.8348419057289813</v>
       </c>
       <c r="AX84" t="n">
-        <v>0.05401231484169378</v>
+        <v>0.06353649806574668</v>
       </c>
       <c r="AY84" t="n">
-        <v>7.222928080519338</v>
+        <v>7.297231456840741</v>
       </c>
       <c r="AZ84" t="inlineStr"/>
       <c r="BA84" t="n">
@@ -16783,10 +16783,10 @@
         </is>
       </c>
       <c r="Z85" t="n">
-        <v>0.1476428806781769</v>
+        <v>0.1477825343608856</v>
       </c>
       <c r="AA85" t="n">
-        <v>28523875980.19678</v>
+        <v>28550856382.55322</v>
       </c>
       <c r="AB85" t="inlineStr">
         <is>
@@ -16854,13 +16854,13 @@
         <v>3.811417863679924</v>
       </c>
       <c r="AW85" t="n">
-        <v>9.551426845298769</v>
+        <v>9.551425935681793</v>
       </c>
       <c r="AX85" t="n">
         <v>2.295919679701158</v>
       </c>
       <c r="AY85" t="n">
-        <v>25.81189019778624</v>
+        <v>25.8118813876588</v>
       </c>
       <c r="AZ85" t="inlineStr"/>
       <c r="BA85" t="n">
@@ -16975,10 +16975,10 @@
         </is>
       </c>
       <c r="Z86" t="n">
-        <v>0.1476428806781769</v>
+        <v>0.1477825343608856</v>
       </c>
       <c r="AA86" t="n">
-        <v>107670922721.084</v>
+        <v>107772767393.916</v>
       </c>
       <c r="AB86" t="inlineStr">
         <is>
@@ -17388,16 +17388,16 @@
         <v>405.9760382080078</v>
       </c>
       <c r="AG88" t="n">
-        <v>361.2549255371094</v>
+        <v>361.2549252319336</v>
       </c>
       <c r="AH88" t="n">
         <v>-0.0147940676839341</v>
       </c>
       <c r="AI88" t="n">
-        <v>0.1071682984696545</v>
+        <v>0.1071682994049523</v>
       </c>
       <c r="AJ88" t="n">
-        <v>0.1237937797094604</v>
+        <v>0.1237937806588028</v>
       </c>
       <c r="AK88" t="n">
         <v>480.8090515136719</v>
@@ -17436,13 +17436,13 @@
         <v>0.4629652450487607</v>
       </c>
       <c r="AW88" t="n">
-        <v>8.384254085964638</v>
+        <v>8.384253246055829</v>
       </c>
       <c r="AX88" t="n">
         <v>0.154834014083173</v>
       </c>
       <c r="AY88" t="n">
-        <v>351.2130314740801</v>
+        <v>351.2129205528598</v>
       </c>
       <c r="AZ88" t="inlineStr"/>
       <c r="BA88" t="n">
@@ -17974,28 +17974,28 @@
         <v>190.6975485229492</v>
       </c>
       <c r="AG91" t="n">
-        <v>129.671023979187</v>
+        <v>129.6710235977173</v>
       </c>
       <c r="AH91" t="n">
         <v>0.001009194235530808</v>
       </c>
       <c r="AI91" t="n">
-        <v>0.4721099096147143</v>
+        <v>0.472109913945407</v>
       </c>
       <c r="AJ91" t="n">
-        <v>0.470625762572503</v>
+        <v>0.4706257668988294</v>
       </c>
       <c r="AK91" t="n">
         <v>255.6900024414062</v>
       </c>
       <c r="AL91" t="n">
-        <v>51.04203796386719</v>
+        <v>51.04204177856445</v>
       </c>
       <c r="AM91" t="n">
         <v>-0.253431899695051</v>
       </c>
       <c r="AN91" t="n">
-        <v>2.739858497123098</v>
+        <v>2.739858217619624</v>
       </c>
       <c r="AO91" t="n">
         <v>48.92653588973677</v>
@@ -18022,13 +18022,13 @@
         <v>2.692627270706699</v>
       </c>
       <c r="AW91" t="n">
-        <v>4.271910426759877</v>
+        <v>4.271909871350892</v>
       </c>
       <c r="AX91" t="n">
-        <v>1.112489314214237</v>
+        <v>1.112489135854879</v>
       </c>
       <c r="AY91" t="n">
-        <v>248.0077526202706</v>
+        <v>248.0077332595004</v>
       </c>
       <c r="AZ91" t="inlineStr"/>
       <c r="BA91" t="n">
@@ -18170,28 +18170,28 @@
         <v>93.51835311889648</v>
       </c>
       <c r="AG92" t="n">
-        <v>73.68087131500243</v>
+        <v>73.68087148666382</v>
       </c>
       <c r="AH92" t="n">
         <v>-0.05269935383421576</v>
       </c>
       <c r="AI92" t="n">
-        <v>0.2023472952586065</v>
+        <v>0.2023472924573828</v>
       </c>
       <c r="AJ92" t="n">
-        <v>0.269235168502342</v>
+        <v>0.2692351655452832</v>
       </c>
       <c r="AK92" t="n">
         <v>102.7099990844727</v>
       </c>
       <c r="AL92" t="n">
-        <v>48.05623245239258</v>
+        <v>48.05623626708984</v>
       </c>
       <c r="AM92" t="n">
         <v>-0.1374744705719372</v>
       </c>
       <c r="AN92" t="n">
-        <v>0.8434652867482537</v>
+        <v>0.843465140414239</v>
       </c>
       <c r="AO92" t="n">
         <v>36.58184653775317</v>
@@ -18212,19 +18212,19 @@
         <v>0.24419557916485</v>
       </c>
       <c r="AU92" t="n">
-        <v>0.2179910775302019</v>
+        <v>0.2179909497705974</v>
       </c>
       <c r="AV92" t="n">
         <v>0.2119475223825824</v>
       </c>
       <c r="AW92" t="n">
-        <v>0.3290019358750822</v>
+        <v>0.3290020879846971</v>
       </c>
       <c r="AX92" t="n">
         <v>0.3771933486728183</v>
       </c>
       <c r="AY92" t="n">
-        <v>503.2814332234295</v>
+        <v>503.2812193527712</v>
       </c>
       <c r="AZ92" t="inlineStr"/>
       <c r="BA92" t="n">
@@ -18420,7 +18420,7 @@
         <v>1.641861886780454</v>
       </c>
       <c r="AY93" t="n">
-        <v>18.44134625341344</v>
+        <v>18.44135083917955</v>
       </c>
       <c r="AZ93" t="inlineStr"/>
       <c r="BA93" t="n">
@@ -18552,67 +18552,67 @@
         <v>25.2</v>
       </c>
       <c r="AE94" t="n">
-        <v>939.5</v>
+        <v>936.5</v>
       </c>
       <c r="AF94" t="n">
-        <v>995.65</v>
+        <v>996.13</v>
       </c>
       <c r="AG94" t="n">
-        <v>833.88</v>
+        <v>835.4025</v>
       </c>
       <c r="AH94" t="n">
-        <v>-0.05639531964043587</v>
+        <v>-0.05986166464216514</v>
       </c>
       <c r="AI94" t="n">
-        <v>0.1266609104427496</v>
+        <v>0.1210165159907948</v>
       </c>
       <c r="AJ94" t="n">
-        <v>0.1939967381397802</v>
+        <v>0.1923952825135189</v>
       </c>
       <c r="AK94" t="n">
         <v>1112</v>
       </c>
       <c r="AL94" t="n">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="AM94" t="n">
-        <v>-0.1551258992805755</v>
+        <v>-0.1578237410071942</v>
       </c>
       <c r="AN94" t="n">
-        <v>0.8640873015873016</v>
+        <v>0.8507905138339922</v>
       </c>
       <c r="AO94" t="n">
-        <v>32.45778611632271</v>
+        <v>23.59081419624218</v>
       </c>
       <c r="AP94" t="n">
-        <v>119831</v>
+        <v>122555</v>
       </c>
       <c r="AQ94" t="n">
-        <v>147696.82</v>
+        <v>147751.3</v>
       </c>
       <c r="AR94" t="n">
-        <v>0.8113309413161366</v>
+        <v>0.8294681671159577</v>
       </c>
       <c r="AS94" t="n">
-        <v>-0.04327902240325865</v>
+        <v>-0.04487506374298822</v>
       </c>
       <c r="AT94" t="n">
-        <v>0.03526170798898076</v>
+        <v>0.02126499454743724</v>
       </c>
       <c r="AU94" t="n">
-        <v>0.1380981223500908</v>
+        <v>0.1469687691365584</v>
       </c>
       <c r="AV94" t="n">
-        <v>0.8640873015873016</v>
+        <v>0.8507905138339922</v>
       </c>
       <c r="AW94" t="n">
-        <v>2.54061155078386</v>
+        <v>2.544021081724945</v>
       </c>
       <c r="AX94" t="n">
-        <v>0.1401699029126213</v>
+        <v>0.1365291262135921</v>
       </c>
       <c r="AY94" t="n">
-        <v>26.81621423939938</v>
+        <v>26.72739497324481</v>
       </c>
       <c r="AZ94" t="inlineStr"/>
       <c r="BA94" t="n">
@@ -18798,13 +18798,13 @@
         <v>1.485924787553267</v>
       </c>
       <c r="AW95" t="n">
-        <v>1.569356231173189</v>
+        <v>1.569356484218569</v>
       </c>
       <c r="AX95" t="n">
         <v>0.9109061663612272</v>
       </c>
       <c r="AY95" t="n">
-        <v>19.81849540221389</v>
+        <v>19.81849124896149</v>
       </c>
       <c r="AZ95" t="inlineStr"/>
       <c r="BA95" t="n">
@@ -18936,22 +18936,22 @@
         <v>19.2</v>
       </c>
       <c r="AE96" t="n">
-        <v>136.5500030517578</v>
+        <v>135.0500030517578</v>
       </c>
       <c r="AF96" t="n">
-        <v>146.0310006713867</v>
+        <v>146.173000793457</v>
       </c>
       <c r="AG96" t="n">
-        <v>107.1124338150024</v>
+        <v>107.3725777816773</v>
       </c>
       <c r="AH96" t="n">
-        <v>-0.06492455421136212</v>
+        <v>-0.07609474856041332</v>
       </c>
       <c r="AI96" t="n">
-        <v>0.2748286841058807</v>
+        <v>0.2577699617714089</v>
       </c>
       <c r="AJ96" t="n">
-        <v>0.3633431289928661</v>
+        <v>0.3613624988185851</v>
       </c>
       <c r="AK96" t="n">
         <v>156.8999938964844</v>
@@ -18960,13 +18960,13 @@
         <v>60.389892578125</v>
       </c>
       <c r="AM96" t="n">
-        <v>-0.1297003928384636</v>
+        <v>-0.1392606226558697</v>
       </c>
       <c r="AN96" t="n">
-        <v>1.261140022315924</v>
+        <v>1.236301428704262</v>
       </c>
       <c r="AO96" t="n">
-        <v>29.86699946935585</v>
+        <v>26.2394304763915</v>
       </c>
       <c r="AP96" t="n">
         <v>588526</v>
@@ -18978,25 +18978,25 @@
         <v>0.5216668961249582</v>
       </c>
       <c r="AS96" t="n">
-        <v>-0.0447708571746358</v>
+        <v>-0.06150098137664184</v>
       </c>
       <c r="AT96" t="n">
-        <v>0.1492712019877682</v>
+        <v>0.1152179117567009</v>
       </c>
       <c r="AU96" t="n">
-        <v>0.6037277193233976</v>
+        <v>0.5769191640328666</v>
       </c>
       <c r="AV96" t="n">
-        <v>1.243440325510321</v>
+        <v>1.226785420008177</v>
       </c>
       <c r="AW96" t="n">
-        <v>3.91501631415559</v>
+        <v>3.830330546155774</v>
       </c>
       <c r="AX96" t="n">
-        <v>0.5305715248879002</v>
+        <v>0.5137582166782941</v>
       </c>
       <c r="AY96" t="n">
-        <v>12.04192381667881</v>
+        <v>11.89865492924968</v>
       </c>
       <c r="AZ96" t="inlineStr"/>
       <c r="BA96" t="n">
@@ -19918,28 +19918,28 @@
         <v>206.4163836669922</v>
       </c>
       <c r="AG101" t="n">
-        <v>219.7730899810791</v>
+        <v>219.7730899047852</v>
       </c>
       <c r="AH101" t="n">
         <v>-0.02934061215998851</v>
       </c>
       <c r="AI101" t="n">
-        <v>-0.08833242219235693</v>
+        <v>-0.08833242187587276</v>
       </c>
       <c r="AJ101" t="n">
-        <v>-0.06077498530523839</v>
+        <v>-0.06077498497918776</v>
       </c>
       <c r="AK101" t="n">
-        <v>247.2834320068359</v>
+        <v>247.2834167480469</v>
       </c>
       <c r="AL101" t="n">
-        <v>173.2072296142578</v>
+        <v>173.2072143554688</v>
       </c>
       <c r="AM101" t="n">
-        <v>-0.1897556622199712</v>
+        <v>-0.189755612223301</v>
       </c>
       <c r="AN101" t="n">
-        <v>0.1567646515481167</v>
+        <v>0.1567647534539631</v>
       </c>
       <c r="AO101" t="n">
         <v>29.29049506978377</v>
@@ -19963,16 +19963,16 @@
         <v>-0.1152442960791923</v>
       </c>
       <c r="AV101" t="n">
-        <v>0.1567646515481167</v>
+        <v>0.1567647534539631</v>
       </c>
       <c r="AW101" t="n">
-        <v>0.5652151057380206</v>
+        <v>0.5652156654679326</v>
       </c>
       <c r="AX101" t="n">
         <v>-0.1349333530448573</v>
       </c>
       <c r="AY101" t="n">
-        <v>6.49762173299658</v>
+        <v>6.497619592443621</v>
       </c>
       <c r="AZ101" t="inlineStr"/>
       <c r="BA101" t="n">
@@ -20110,16 +20110,16 @@
         <v>68.33011245727539</v>
       </c>
       <c r="AG102" t="n">
-        <v>39.5800168800354</v>
+        <v>39.58001675605774</v>
       </c>
       <c r="AH102" t="n">
         <v>0.04580537796062134</v>
       </c>
       <c r="AI102" t="n">
-        <v>0.8054565085473187</v>
+        <v>0.8054565142026038</v>
       </c>
       <c r="AJ102" t="n">
-        <v>0.7263790630605278</v>
+        <v>0.7263790684681162</v>
       </c>
       <c r="AK102" t="n">
         <v>79.81999969482422</v>
@@ -20155,16 +20155,16 @@
         <v>1.558649224932994</v>
       </c>
       <c r="AV102" t="n">
-        <v>1.179157582388999</v>
+        <v>1.179157835886916</v>
       </c>
       <c r="AW102" t="n">
-        <v>1.001995282711361</v>
+        <v>1.001995068756024</v>
       </c>
       <c r="AX102" t="n">
         <v>1.621283151616665</v>
       </c>
       <c r="AY102" t="n">
-        <v>31.63501736469518</v>
+        <v>31.63502802491553</v>
       </c>
       <c r="AZ102" t="inlineStr"/>
       <c r="BA102" t="n">
@@ -20492,16 +20492,16 @@
         <v>24019.4</v>
       </c>
       <c r="AG104" t="n">
-        <v>20367.691328125</v>
+        <v>20367.69135742187</v>
       </c>
       <c r="AH104" t="n">
         <v>0.04540496432050745</v>
       </c>
       <c r="AI104" t="n">
-        <v>0.2328348655464214</v>
+        <v>0.2328348637731126</v>
       </c>
       <c r="AJ104" t="n">
-        <v>0.1792892779572168</v>
+        <v>0.1792892762609282</v>
       </c>
       <c r="AK104" t="n">
         <v>26150</v>
@@ -20537,7 +20537,7 @@
         <v>0.2472633118227161</v>
       </c>
       <c r="AV104" t="n">
-        <v>0.5024855957921166</v>
+        <v>0.5024857713838278</v>
       </c>
       <c r="AW104" t="n">
         <v>0.2956386056429623</v>
@@ -20546,7 +20546,7 @@
         <v>0.2512668323366565</v>
       </c>
       <c r="AY104" t="n">
-        <v>22.41635869067181</v>
+        <v>22.41636402196004</v>
       </c>
       <c r="AZ104" t="inlineStr"/>
       <c r="BA104" t="n">
@@ -20688,28 +20688,28 @@
         <v>405.4028820800781</v>
       </c>
       <c r="AG105" t="n">
-        <v>370.6051461791992</v>
+        <v>370.6051469421387</v>
       </c>
       <c r="AH105" t="n">
         <v>0.004630250011019799</v>
       </c>
       <c r="AI105" t="n">
-        <v>0.09895937220030993</v>
+        <v>0.0989593699379574</v>
       </c>
       <c r="AJ105" t="n">
-        <v>0.09389436779178761</v>
+        <v>0.09389436553986208</v>
       </c>
       <c r="AK105" t="n">
         <v>435.7799987792969</v>
       </c>
       <c r="AL105" t="n">
-        <v>313.9706420898438</v>
+        <v>313.9706115722656</v>
       </c>
       <c r="AM105" t="n">
         <v>-0.06539997264636732</v>
       </c>
       <c r="AN105" t="n">
-        <v>0.2971913426948765</v>
+        <v>0.2971914687803656</v>
       </c>
       <c r="AO105" t="n">
         <v>45.81093261114604</v>
@@ -20733,7 +20733,7 @@
         <v>0.2779306941870878</v>
       </c>
       <c r="AV105" t="n">
-        <v>0.1520144487025483</v>
+        <v>0.1520145481452402</v>
       </c>
       <c r="AW105" t="n">
         <v>1.913155524064541</v>
@@ -20742,7 +20742,7 @@
         <v>0.2516544918972008</v>
       </c>
       <c r="AY105" t="n">
-        <v>1178.185307538381</v>
+        <v>1178.185918020038</v>
       </c>
       <c r="AZ105" t="inlineStr"/>
       <c r="BA105" t="n">
@@ -20874,22 +20874,22 @@
         <v>26.5</v>
       </c>
       <c r="AE106" t="n">
-        <v>270</v>
+        <v>269.6499938964844</v>
       </c>
       <c r="AF106" t="n">
-        <v>272.7169253540039</v>
+        <v>272.8206924438476</v>
       </c>
       <c r="AG106" t="n">
-        <v>249.4604872894287</v>
+        <v>249.6712863922119</v>
       </c>
       <c r="AH106" t="n">
-        <v>-0.009962437609903341</v>
+        <v>-0.01162191371541899</v>
       </c>
       <c r="AI106" t="n">
-        <v>0.08233573554572993</v>
+        <v>0.08002004472748081</v>
       </c>
       <c r="AJ106" t="n">
-        <v>0.09322694073628046</v>
+        <v>0.09271953690049073</v>
       </c>
       <c r="AK106" t="n">
         <v>292.75</v>
@@ -20898,13 +20898,13 @@
         <v>206.813720703125</v>
       </c>
       <c r="AM106" t="n">
-        <v>-0.07771135781383431</v>
+        <v>-0.07890693801371695</v>
       </c>
       <c r="AN106" t="n">
-        <v>0.3055226659143038</v>
+        <v>0.3038302922056075</v>
       </c>
       <c r="AO106" t="n">
-        <v>35.79337073215996</v>
+        <v>32.12075689183986</v>
       </c>
       <c r="AP106" t="n">
         <v>643592</v>
@@ -20916,25 +20916,25 @@
         <v>0.6584889291963153</v>
       </c>
       <c r="AS106" t="n">
-        <v>0.02156644899846216</v>
+        <v>0.01639655598819778</v>
       </c>
       <c r="AT106" t="n">
-        <v>0.05349618615843066</v>
+        <v>0.02362012891099896</v>
       </c>
       <c r="AU106" t="n">
-        <v>0.1580449039262368</v>
+        <v>0.1485408113326865</v>
       </c>
       <c r="AV106" t="n">
-        <v>0.2141910055945619</v>
+        <v>0.2305978932784376</v>
       </c>
       <c r="AW106" t="n">
-        <v>1.00120221057459</v>
+        <v>0.9851765960608947</v>
       </c>
       <c r="AX106" t="n">
-        <v>0.1568236382525496</v>
+        <v>0.1553240259041069</v>
       </c>
       <c r="AY106" t="n">
-        <v>13.50897077742911</v>
+        <v>13.49015806885431</v>
       </c>
       <c r="AZ106" t="inlineStr"/>
       <c r="BA106" t="n">
@@ -21076,16 +21076,16 @@
         <v>470.2074084472656</v>
       </c>
       <c r="AG107" t="n">
-        <v>434.4708938598633</v>
+        <v>434.4708941650391</v>
       </c>
       <c r="AH107" t="n">
         <v>0.02018812036822726</v>
       </c>
       <c r="AI107" t="n">
-        <v>0.1041016072339163</v>
+        <v>0.1041016064583866</v>
       </c>
       <c r="AJ107" t="n">
-        <v>0.08225295432317026</v>
+        <v>0.08225295356298745</v>
       </c>
       <c r="AK107" t="n">
         <v>503.4599914550781</v>
@@ -21118,19 +21118,19 @@
         <v>0.03237760243543963</v>
       </c>
       <c r="AU107" t="n">
-        <v>0.2737823113022542</v>
+        <v>0.2737824145239043</v>
       </c>
       <c r="AV107" t="n">
         <v>0.1116547221922246</v>
       </c>
       <c r="AW107" t="n">
-        <v>1.722768135450301</v>
+        <v>1.722767663820131</v>
       </c>
       <c r="AX107" t="n">
         <v>0.2109252523683778</v>
       </c>
       <c r="AY107" t="n">
-        <v>537.0775834311247</v>
+        <v>537.0777992808987</v>
       </c>
       <c r="AZ107" t="inlineStr"/>
       <c r="BA107" t="n">
@@ -21272,16 +21272,16 @@
         <v>299.4725476074219</v>
       </c>
       <c r="AG108" t="n">
-        <v>217.126110534668</v>
+        <v>217.1261102294922</v>
       </c>
       <c r="AH108" t="n">
         <v>0.04002852329346251</v>
       </c>
       <c r="AI108" t="n">
-        <v>0.4344658534531622</v>
+        <v>0.4344658554693372</v>
       </c>
       <c r="AJ108" t="n">
-        <v>0.3792562620404232</v>
+        <v>0.3792562639789998</v>
       </c>
       <c r="AK108" t="n">
         <v>332.2799987792969</v>
@@ -21326,7 +21326,7 @@
         <v>0.7749315156521179</v>
       </c>
       <c r="AY108" t="n">
-        <v>451.9822104087669</v>
+        <v>451.9821711406484</v>
       </c>
       <c r="AZ108" t="inlineStr"/>
       <c r="BA108" t="n">
@@ -21518,7 +21518,7 @@
         <v>0.3014092246636779</v>
       </c>
       <c r="AY109" t="n">
-        <v>54.94409013938794</v>
+        <v>54.94411460459389</v>
       </c>
       <c r="AZ109" t="inlineStr"/>
       <c r="BA109" t="n">
@@ -21704,13 +21704,13 @@
         <v>3.457147487656786</v>
       </c>
       <c r="AW110" t="n">
-        <v>6.426257549583001</v>
+        <v>6.426257997195557</v>
       </c>
       <c r="AX110" t="n">
         <v>0.8993271374731151</v>
       </c>
       <c r="AY110" t="n">
-        <v>75.10735162307959</v>
+        <v>75.10736925285615</v>
       </c>
       <c r="AZ110" t="inlineStr"/>
       <c r="BA110" t="n">
@@ -21852,28 +21852,28 @@
         <v>407.8515246582031</v>
       </c>
       <c r="AG111" t="n">
-        <v>319.6667751312256</v>
+        <v>319.6667750549316</v>
       </c>
       <c r="AH111" t="n">
         <v>-0.02991659960556514</v>
       </c>
       <c r="AI111" t="n">
-        <v>0.2376950771129316</v>
+        <v>0.2376950774083286</v>
       </c>
       <c r="AJ111" t="n">
-        <v>0.2758646077334033</v>
+        <v>0.2758646080379101</v>
       </c>
       <c r="AK111" t="n">
         <v>445.4800109863281</v>
       </c>
       <c r="AL111" t="n">
-        <v>217.7568969726562</v>
+        <v>217.7568817138672</v>
       </c>
       <c r="AM111" t="n">
         <v>-0.1118569090889536</v>
       </c>
       <c r="AN111" t="n">
-        <v>0.816934385991761</v>
+        <v>0.8169345133090624</v>
       </c>
       <c r="AO111" t="n">
         <v>37.81781564690416</v>
@@ -21897,16 +21897,16 @@
         <v>0.3303114170092663</v>
       </c>
       <c r="AV111" t="n">
-        <v>0.6357079710719991</v>
+        <v>0.6357078678860844</v>
       </c>
       <c r="AW111" t="n">
-        <v>1.523124023030024</v>
+        <v>1.523124268549611</v>
       </c>
       <c r="AX111" t="n">
         <v>0.4538465316690081</v>
       </c>
       <c r="AY111" t="n">
-        <v>890.8785904570318</v>
+        <v>890.8788301252961</v>
       </c>
       <c r="AZ111" t="inlineStr"/>
       <c r="BA111" t="n">
@@ -22048,25 +22048,25 @@
         <v>67.81264907836913</v>
       </c>
       <c r="AG112" t="n">
-        <v>60.02419466018677</v>
+        <v>60.02419464111328</v>
       </c>
       <c r="AH112" t="n">
         <v>0.02252304371351688</v>
       </c>
       <c r="AI112" t="n">
-        <v>0.1552007774605413</v>
+        <v>0.1552007778276216</v>
       </c>
       <c r="AJ112" t="n">
-        <v>0.1297552505664576</v>
+        <v>0.1297552509254525</v>
       </c>
       <c r="AK112" t="n">
-        <v>79.79306030273438</v>
+        <v>79.79306793212891</v>
       </c>
       <c r="AL112" t="n">
         <v>49.96692657470703</v>
       </c>
       <c r="AM112" t="n">
-        <v>-0.1310021689252786</v>
+        <v>-0.1310022520142922</v>
       </c>
       <c r="AN112" t="n">
         <v>0.3877178584161733</v>
@@ -22090,19 +22090,19 @@
         <v>0.09862607854849625</v>
       </c>
       <c r="AU112" t="n">
-        <v>0.2975393523804519</v>
+        <v>0.2975394450031381</v>
       </c>
       <c r="AV112" t="n">
-        <v>-0.08348584145152504</v>
+        <v>-0.08348593387548497</v>
       </c>
       <c r="AW112" t="n">
         <v>0.5285008870605208</v>
       </c>
       <c r="AX112" t="n">
-        <v>0.305782288490881</v>
+        <v>0.3057823822941217</v>
       </c>
       <c r="AY112" t="n">
-        <v>5.270668951794295</v>
+        <v>5.270667329367306</v>
       </c>
       <c r="AZ112" t="inlineStr"/>
       <c r="BA112" t="n">
@@ -22234,22 +22234,22 @@
         <v>26.3</v>
       </c>
       <c r="AE113" t="n">
-        <v>73.34999847412109</v>
+        <v>72.48000335693359</v>
       </c>
       <c r="AF113" t="n">
-        <v>74.0086003112793</v>
+        <v>74.31560035705566</v>
       </c>
       <c r="AG113" t="n">
-        <v>47.65660281181336</v>
+        <v>47.85129332542419</v>
       </c>
       <c r="AH113" t="n">
-        <v>-0.008898990582015154</v>
+        <v>-0.02470002248925907</v>
       </c>
       <c r="AI113" t="n">
-        <v>0.5391361143337461</v>
+        <v>0.5146926722338716</v>
       </c>
       <c r="AJ113" t="n">
-        <v>0.5529558538514556</v>
+        <v>0.5530531192052552</v>
       </c>
       <c r="AK113" t="n">
         <v>88</v>
@@ -22258,43 +22258,43 @@
         <v>31.03618240356445</v>
       </c>
       <c r="AM113" t="n">
-        <v>-0.1664772900668058</v>
+        <v>-0.1763635982166637</v>
       </c>
       <c r="AN113" t="n">
-        <v>1.363370517686382</v>
+        <v>1.335338876878407</v>
       </c>
       <c r="AO113" t="n">
-        <v>38.18530434024252</v>
+        <v>29.83822619533856</v>
       </c>
       <c r="AP113" t="n">
-        <v>3699154</v>
+        <v>3700611</v>
       </c>
       <c r="AQ113" t="n">
-        <v>5852464.78</v>
+        <v>5852493.92</v>
       </c>
       <c r="AR113" t="n">
-        <v>0.6320677080606028</v>
+        <v>0.6323135146460775</v>
       </c>
       <c r="AS113" t="n">
-        <v>-0.04814429278500432</v>
+        <v>-0.09467892121920896</v>
       </c>
       <c r="AT113" t="n">
-        <v>0.70859534015139</v>
+        <v>0.6304127853235546</v>
       </c>
       <c r="AU113" t="n">
-        <v>0.7740168747042462</v>
+        <v>0.7171205345503193</v>
       </c>
       <c r="AV113" t="n">
-        <v>0.9461403778849484</v>
+        <v>0.9552328380197033</v>
       </c>
       <c r="AW113" t="n">
-        <v>1.386862455077032</v>
+        <v>1.268544110126878</v>
       </c>
       <c r="AX113" t="n">
-        <v>0.9316455139229178</v>
+        <v>0.9087345091484189</v>
       </c>
       <c r="AY113" t="n">
-        <v>0.451825868137077</v>
+        <v>0.4346061605423841</v>
       </c>
       <c r="AZ113" t="inlineStr"/>
       <c r="BA113" t="n">
@@ -22486,7 +22486,7 @@
         <v>0.7463959088542806</v>
       </c>
       <c r="AY114" t="n">
-        <v>277.5895089070024</v>
+        <v>277.5894148473691</v>
       </c>
       <c r="AZ114" t="inlineStr"/>
       <c r="BA114" t="n">
@@ -22628,28 +22628,28 @@
         <v>1516.832399902344</v>
       </c>
       <c r="AG115" t="n">
-        <v>1176.413474731445</v>
+        <v>1176.413475036621</v>
       </c>
       <c r="AH115" t="n">
         <v>-0.1081809761437936</v>
       </c>
       <c r="AI115" t="n">
-        <v>0.1498848145573832</v>
+        <v>0.1498848142590894</v>
       </c>
       <c r="AJ115" t="n">
-        <v>0.2893701342962005</v>
+        <v>0.2893701339617225</v>
       </c>
       <c r="AK115" t="n">
         <v>1687.3154296875</v>
       </c>
       <c r="AL115" t="n">
-        <v>706.2978515625</v>
+        <v>706.2977905273438</v>
       </c>
       <c r="AM115" t="n">
         <v>-0.1982886149005881</v>
       </c>
       <c r="AN115" t="n">
-        <v>0.9152542900163014</v>
+        <v>0.9152544555241742</v>
       </c>
       <c r="AO115" t="n">
         <v>35.08824170085371</v>
@@ -22676,13 +22676,13 @@
         <v>0.8396994829103939</v>
       </c>
       <c r="AW115" t="n">
-        <v>2.727947675193613</v>
+        <v>2.727947361666347</v>
       </c>
       <c r="AX115" t="n">
         <v>0.4498539207849714</v>
       </c>
       <c r="AY115" t="n">
-        <v>160.1430990241444</v>
+        <v>160.1431173308092</v>
       </c>
       <c r="AZ115" t="inlineStr"/>
       <c r="BA115" t="n">
@@ -23219,13 +23219,13 @@
         <v>184.3399963378906</v>
       </c>
       <c r="AL118" t="n">
-        <v>73.89095306396484</v>
+        <v>73.89094543457031</v>
       </c>
       <c r="AM118" t="n">
         <v>-0.1281327741478991</v>
       </c>
       <c r="AN118" t="n">
-        <v>1.175097147299932</v>
+        <v>1.175097371883258</v>
       </c>
       <c r="AO118" t="n">
         <v>39.49742360530085</v>
@@ -23249,16 +23249,16 @@
         <v>0.569901672349572</v>
       </c>
       <c r="AV118" t="n">
-        <v>1.169562933713982</v>
+        <v>1.169562710272086</v>
       </c>
       <c r="AW118" t="n">
         <v>4.500466991153932</v>
       </c>
       <c r="AX118" t="n">
-        <v>0.5096451599056084</v>
+        <v>0.5096452680913273</v>
       </c>
       <c r="AY118" t="n">
-        <v>7.404463173433207</v>
+        <v>7.404462335170647</v>
       </c>
       <c r="AZ118" t="inlineStr"/>
       <c r="BA118" t="n">
@@ -23596,28 +23596,28 @@
         <v>76.80261856079102</v>
       </c>
       <c r="AG120" t="n">
-        <v>51.9581580734253</v>
+        <v>51.95815791130066</v>
       </c>
       <c r="AH120" t="n">
         <v>-0.06162054047962995</v>
       </c>
       <c r="AI120" t="n">
-        <v>0.3870776479985614</v>
+        <v>0.3870776523266488</v>
       </c>
       <c r="AJ120" t="n">
-        <v>0.4781628411895678</v>
+        <v>0.4781628458018679</v>
       </c>
       <c r="AK120" t="n">
         <v>87.34999847412109</v>
       </c>
       <c r="AL120" t="n">
-        <v>30.51562881469727</v>
+        <v>30.51562690734863</v>
       </c>
       <c r="AM120" t="n">
         <v>-0.1749284378502174</v>
       </c>
       <c r="AN120" t="n">
-        <v>1.36174060618122</v>
+        <v>1.361740753799446</v>
       </c>
       <c r="AO120" t="n">
         <v>33.27401999356185</v>
@@ -23644,13 +23644,13 @@
         <v>0.2497011302380263</v>
       </c>
       <c r="AW120" t="n">
-        <v>-0.08558284376219083</v>
+        <v>-0.08558275524567183</v>
       </c>
       <c r="AX120" t="n">
         <v>0.9455866098638481</v>
       </c>
       <c r="AY120" t="n">
-        <v>40.30864236165512</v>
+        <v>40.30863671661076</v>
       </c>
       <c r="AZ120" t="inlineStr"/>
       <c r="BA120" t="n">
@@ -23837,10 +23837,10 @@
         <v>0.5944768253767467</v>
       </c>
       <c r="AV121" t="n">
-        <v>0.7341175920367033</v>
+        <v>0.7341177313882654</v>
       </c>
       <c r="AW121" t="n">
-        <v>6.414155878825276</v>
+        <v>6.414155242003194</v>
       </c>
       <c r="AX121" t="n">
         <v>0.4983397216186964</v>
@@ -24038,7 +24038,7 @@
         <v>1.327999198802591</v>
       </c>
       <c r="AY122" t="n">
-        <v>127.9867750897095</v>
+        <v>127.9867313472839</v>
       </c>
       <c r="AZ122" t="inlineStr"/>
       <c r="BA122" t="n">
@@ -24226,13 +24226,13 @@
         <v>1.644228207456331</v>
       </c>
       <c r="AW123" t="n">
-        <v>10.8881064438188</v>
+        <v>10.88810559843212</v>
       </c>
       <c r="AX123" t="n">
         <v>0.8165378176623308</v>
       </c>
       <c r="AY123" t="n">
-        <v>31.08766645380388</v>
+        <v>31.0876695332767</v>
       </c>
       <c r="AZ123" t="inlineStr"/>
       <c r="BA123" t="n">
@@ -24364,22 +24364,22 @@
         <v>20.3</v>
       </c>
       <c r="AE124" t="n">
-        <v>141.3500061035156</v>
+        <v>140.6999969482422</v>
       </c>
       <c r="AF124" t="n">
-        <v>146.5197937011719</v>
+        <v>146.3463369750976</v>
       </c>
       <c r="AG124" t="n">
-        <v>138.3345943832397</v>
+        <v>138.3392007064819</v>
       </c>
       <c r="AH124" t="n">
-        <v>-0.03528388531722926</v>
+        <v>-0.03858203863220877</v>
       </c>
       <c r="AI124" t="n">
-        <v>0.0217979583033443</v>
+        <v>0.01706527310916894</v>
       </c>
       <c r="AJ124" t="n">
-        <v>0.05916957616007457</v>
+        <v>0.05788045780027806</v>
       </c>
       <c r="AK124" t="n">
         <v>157.5401306152344</v>
@@ -24388,13 +24388,13 @@
         <v>109.7664031982422</v>
       </c>
       <c r="AM124" t="n">
-        <v>-0.1027682562436135</v>
+        <v>-0.1068942472069001</v>
       </c>
       <c r="AN124" t="n">
-        <v>0.2877346982776896</v>
+        <v>0.2818129486682075</v>
       </c>
       <c r="AO124" t="n">
-        <v>33.49592850443869</v>
+        <v>26.86305476455431</v>
       </c>
       <c r="AP124" t="n">
         <v>504696</v>
@@ -24406,25 +24406,25 @@
         <v>0.8360170737673056</v>
       </c>
       <c r="AS124" t="n">
-        <v>0.05682247554030373</v>
+        <v>0.05353795382328341</v>
       </c>
       <c r="AT124" t="n">
-        <v>-0.02446988308715459</v>
+        <v>-0.04196822538484479</v>
       </c>
       <c r="AU124" t="n">
-        <v>0.1333081433086076</v>
+        <v>0.1254327817754612</v>
       </c>
       <c r="AV124" t="n">
-        <v>0.264496557157895</v>
+        <v>0.2818129486682075</v>
       </c>
       <c r="AW124" t="n">
-        <v>0.6417862912691255</v>
+        <v>0.6209334560339062</v>
       </c>
       <c r="AX124" t="n">
-        <v>0.1239969311720819</v>
+        <v>0.1188281426031867</v>
       </c>
       <c r="AY124" t="n">
-        <v>9.439024493313735</v>
+        <v>9.391019815565024</v>
       </c>
       <c r="AZ124" t="inlineStr"/>
       <c r="BA124" t="n">
@@ -24539,10 +24539,10 @@
         </is>
       </c>
       <c r="Z125" t="n">
-        <v>0.1036290898919106</v>
+        <v>0.1035312414169312</v>
       </c>
       <c r="AA125" t="n">
-        <v>3111781235.35556</v>
+        <v>3108843034.811035</v>
       </c>
       <c r="AB125" t="inlineStr">
         <is>
@@ -24556,22 +24556,22 @@
         <v>9.1</v>
       </c>
       <c r="AE125" t="n">
-        <v>163.3500061035156</v>
+        <v>164.5</v>
       </c>
       <c r="AF125" t="n">
-        <v>191.6571319580078</v>
+        <v>191.1065481567383</v>
       </c>
       <c r="AG125" t="n">
-        <v>170.4853285980224</v>
+        <v>170.6139610671997</v>
       </c>
       <c r="AH125" t="n">
-        <v>-0.1476966996495299</v>
+        <v>-0.1392236342153834</v>
       </c>
       <c r="AI125" t="n">
-        <v>-0.04185300021523142</v>
+        <v>-0.03583505727759062</v>
       </c>
       <c r="AJ125" t="n">
-        <v>0.1241854858367617</v>
+        <v>0.1201108453338537</v>
       </c>
       <c r="AK125" t="n">
         <v>210.6000061035156</v>
@@ -24580,43 +24580,43 @@
         <v>110.4240570068359</v>
       </c>
       <c r="AM125" t="n">
-        <v>-0.2243589678567024</v>
+        <v>-0.2188984082025915</v>
       </c>
       <c r="AN125" t="n">
-        <v>0.4792972702805445</v>
+        <v>0.4897116122967338</v>
       </c>
       <c r="AO125" t="n">
-        <v>33.94738772348092</v>
+        <v>37.54579030972526</v>
       </c>
       <c r="AP125" t="n">
-        <v>233500</v>
+        <v>229757</v>
       </c>
       <c r="AQ125" t="n">
-        <v>427990.12</v>
+        <v>427915.26</v>
       </c>
       <c r="AR125" t="n">
-        <v>0.5455733417397579</v>
+        <v>0.5369217260445445</v>
       </c>
       <c r="AS125" t="n">
-        <v>-0.1590733276524292</v>
+        <v>-0.1463414498953859</v>
       </c>
       <c r="AT125" t="n">
-        <v>-0.0893631985311818</v>
+        <v>-0.1391175226975724</v>
       </c>
       <c r="AU125" t="n">
-        <v>-0.0448124941557223</v>
+        <v>-0.01690292658327586</v>
       </c>
       <c r="AV125" t="n">
-        <v>0.2325633822276465</v>
+        <v>0.2477735054937384</v>
       </c>
       <c r="AW125" t="n">
-        <v>1.157943873897437</v>
+        <v>1.115560280928108</v>
       </c>
       <c r="AX125" t="n">
-        <v>-0.1515483858798228</v>
+        <v>-0.1455752353365518</v>
       </c>
       <c r="AY125" t="n">
-        <v>1.618313189244213</v>
+        <v>1.636746272037043</v>
       </c>
       <c r="AZ125" t="inlineStr"/>
       <c r="BA125" t="n">
@@ -25110,22 +25110,22 @@
         <v>29.7</v>
       </c>
       <c r="AE128" t="n">
-        <v>273.7999877929688</v>
+        <v>272.8500061035156</v>
       </c>
       <c r="AF128" t="n">
-        <v>269.2169982910156</v>
+        <v>269.6229983520508</v>
       </c>
       <c r="AG128" t="n">
-        <v>242.9978480529785</v>
+        <v>243.2409336853027</v>
       </c>
       <c r="AH128" t="n">
-        <v>0.01702340316936102</v>
+        <v>0.01196859233518088</v>
       </c>
       <c r="AI128" t="n">
-        <v>0.1267588992527815</v>
+        <v>0.1217273423909815</v>
       </c>
       <c r="AJ128" t="n">
-        <v>0.107898693128841</v>
+        <v>0.1084606290028483</v>
       </c>
       <c r="AK128" t="n">
         <v>284.1000061035156</v>
@@ -25134,43 +25134,43 @@
         <v>203.75</v>
       </c>
       <c r="AM128" t="n">
-        <v>-0.03625490351729854</v>
+        <v>-0.03959873198982233</v>
       </c>
       <c r="AN128" t="n">
-        <v>0.3438036210697852</v>
+        <v>0.3391411342503834</v>
       </c>
       <c r="AO128" t="n">
-        <v>49.5442628136099</v>
+        <v>45.80205019883304</v>
       </c>
       <c r="AP128" t="n">
-        <v>645459</v>
+        <v>645662</v>
       </c>
       <c r="AQ128" t="n">
-        <v>1068654.3</v>
+        <v>1068658.36</v>
       </c>
       <c r="AR128" t="n">
-        <v>0.6039923294184096</v>
+        <v>0.6041799925656315</v>
       </c>
       <c r="AS128" t="n">
-        <v>0.05918757366719052</v>
+        <v>0.03156902118531435</v>
       </c>
       <c r="AT128" t="n">
-        <v>0.1972015367142015</v>
+        <v>0.1500527127650817</v>
       </c>
       <c r="AU128" t="n">
-        <v>0.08233356557818805</v>
+        <v>0.06456815076546629</v>
       </c>
       <c r="AV128" t="n">
-        <v>0.2536241821971628</v>
+        <v>0.2648693162751559</v>
       </c>
       <c r="AW128" t="n">
-        <v>1.367685404961981</v>
+        <v>1.297994897542174</v>
       </c>
       <c r="AX128" t="n">
-        <v>0.1597713388967867</v>
+        <v>0.1557473740135686</v>
       </c>
       <c r="AY128" t="n">
-        <v>27.80212166529779</v>
+        <v>27.70218639208188</v>
       </c>
       <c r="AZ128" t="inlineStr"/>
       <c r="BA128" t="n">
@@ -25302,22 +25302,22 @@
         <v>28</v>
       </c>
       <c r="AE129" t="n">
-        <v>254.8000030517578</v>
+        <v>255.3000030517578</v>
       </c>
       <c r="AF129" t="n">
-        <v>276.9779989624024</v>
+        <v>277.1399990844727</v>
       </c>
       <c r="AG129" t="n">
-        <v>190.6347431945801</v>
+        <v>191.2817120361328</v>
       </c>
       <c r="AH129" t="n">
-        <v>-0.08007132694194619</v>
+        <v>-0.0788049220785989</v>
       </c>
       <c r="AI129" t="n">
-        <v>0.3365874382702871</v>
+        <v>0.334680667242941</v>
       </c>
       <c r="AJ129" t="n">
-        <v>0.4529250771444746</v>
+        <v>0.448857792699604</v>
       </c>
       <c r="AK129" t="n">
         <v>320.2999877929688</v>
@@ -25326,13 +25326,13 @@
         <v>105.1371765136719</v>
       </c>
       <c r="AM129" t="n">
-        <v>-0.2044957453559066</v>
+        <v>-0.2029347087681588</v>
       </c>
       <c r="AN129" t="n">
-        <v>1.423500530458168</v>
+        <v>1.428256222179973</v>
       </c>
       <c r="AO129" t="n">
-        <v>30.57910436309706</v>
+        <v>25.30396117404072</v>
       </c>
       <c r="AP129" t="n">
         <v>286489</v>
@@ -25344,25 +25344,25 @@
         <v>0.6751865518979857</v>
       </c>
       <c r="AS129" t="n">
-        <v>-0.1724585641355314</v>
+        <v>-0.1946372143477672</v>
       </c>
       <c r="AT129" t="n">
-        <v>0.2392767793861716</v>
+        <v>0.1784839599916688</v>
       </c>
       <c r="AU129" t="n">
-        <v>0.581291233680177</v>
+        <v>0.5365401377228389</v>
       </c>
       <c r="AV129" t="n">
-        <v>1.030137350528242</v>
+        <v>1.14180506156428</v>
       </c>
       <c r="AW129" t="n">
-        <v>2.73421332633239</v>
+        <v>2.780996602573403</v>
       </c>
       <c r="AX129" t="n">
-        <v>0.7196938559768227</v>
+        <v>0.7230684514151664</v>
       </c>
       <c r="AY129" t="n">
-        <v>119.9952063100407</v>
+        <v>120.2326517562336</v>
       </c>
       <c r="AZ129" t="inlineStr"/>
       <c r="BA129" t="n">
@@ -25748,13 +25748,13 @@
         <v>1.686475000035968</v>
       </c>
       <c r="AW131" t="n">
-        <v>4.504476840210782</v>
+        <v>4.504477245874732</v>
       </c>
       <c r="AX131" t="n">
         <v>0.9935572470934426</v>
       </c>
       <c r="AY131" t="n">
-        <v>25.91825501891138</v>
+        <v>25.9182525935969</v>
       </c>
       <c r="AZ131" t="inlineStr"/>
       <c r="BA131" t="n">
@@ -25896,28 +25896,28 @@
         <v>1683.27759765625</v>
       </c>
       <c r="AG132" t="n">
-        <v>1333.788044738769</v>
+        <v>1333.788038635254</v>
       </c>
       <c r="AH132" t="n">
         <v>0.06775017310965348</v>
       </c>
       <c r="AI132" t="n">
-        <v>0.3475304066329958</v>
+        <v>0.3475304127993974</v>
       </c>
       <c r="AJ132" t="n">
-        <v>0.2620278044147037</v>
+        <v>0.262027810189839</v>
       </c>
       <c r="AK132" t="n">
         <v>1989.43994140625</v>
       </c>
       <c r="AL132" t="n">
-        <v>686.0034790039062</v>
+        <v>686.00341796875</v>
       </c>
       <c r="AM132" t="n">
         <v>-0.09656988940384204</v>
       </c>
       <c r="AN132" t="n">
-        <v>1.619986634614178</v>
+        <v>1.619986867719859</v>
       </c>
       <c r="AO132" t="n">
         <v>42.68130261249851</v>
@@ -25950,7 +25950,7 @@
         <v>0.5497958659956337</v>
       </c>
       <c r="AY132" t="n">
-        <v>1019.026207960825</v>
+        <v>1019.025793905437</v>
       </c>
       <c r="AZ132" t="inlineStr"/>
       <c r="BA132" t="n">
@@ -26092,16 +26092,16 @@
         <v>423.3733288574219</v>
       </c>
       <c r="AG133" t="n">
-        <v>346.8720091247558</v>
+        <v>346.8720056152344</v>
       </c>
       <c r="AH133" t="n">
         <v>0.02535978476281486</v>
       </c>
       <c r="AI133" t="n">
-        <v>0.2514990369125769</v>
+        <v>0.2514990495747769</v>
       </c>
       <c r="AJ133" t="n">
-        <v>0.2205462468006509</v>
+        <v>0.2205462591496821</v>
       </c>
       <c r="AK133" t="n">
         <v>477.5700073242188</v>
@@ -26134,19 +26134,19 @@
         <v>0.1741139081278711</v>
       </c>
       <c r="AU133" t="n">
-        <v>0.3721351987022659</v>
+        <v>0.3721350663461367</v>
       </c>
       <c r="AV133" t="n">
-        <v>0.9103021558541806</v>
+        <v>0.9103020275843869</v>
       </c>
       <c r="AW133" t="n">
-        <v>2.960454247991606</v>
+        <v>2.960454523655781</v>
       </c>
       <c r="AX133" t="n">
         <v>0.3652661944081437</v>
       </c>
       <c r="AY133" t="n">
-        <v>138.008396437675</v>
+        <v>138.0084070502903</v>
       </c>
       <c r="AZ133" t="inlineStr"/>
       <c r="BA133" t="n">
@@ -26524,13 +26524,13 @@
         <v>0.7165034425969403</v>
       </c>
       <c r="AW135" t="n">
-        <v>6.572757964363883</v>
+        <v>6.572757192553036</v>
       </c>
       <c r="AX135" t="n">
         <v>0.4280315272499267</v>
       </c>
       <c r="AY135" t="n">
-        <v>48.65044641518445</v>
+        <v>48.65044226794548</v>
       </c>
       <c r="AZ135" t="inlineStr"/>
       <c r="BA135" t="n">
@@ -26716,13 +26716,13 @@
         <v>1.809065102870577</v>
       </c>
       <c r="AW136" t="n">
-        <v>12.62433233805926</v>
+        <v>12.62433385726749</v>
       </c>
       <c r="AX136" t="n">
         <v>0.4106542218184528</v>
       </c>
       <c r="AY136" t="n">
-        <v>11.57841765842173</v>
+        <v>11.57842024823771</v>
       </c>
       <c r="AZ136" t="inlineStr"/>
       <c r="BA136" t="n">
@@ -26908,13 +26908,13 @@
         <v>1.305639352180217</v>
       </c>
       <c r="AW137" t="n">
-        <v>1.608889339984027</v>
+        <v>1.608889040444591</v>
       </c>
       <c r="AX137" t="n">
         <v>0.4050945759565934</v>
       </c>
       <c r="AY137" t="n">
-        <v>341.0263403144162</v>
+        <v>341.0263805353297</v>
       </c>
       <c r="AZ137" t="inlineStr"/>
       <c r="BA137" t="n">
@@ -27104,13 +27104,13 @@
         <v>2.064787417039764</v>
       </c>
       <c r="AW138" t="n">
-        <v>3.548506572078137</v>
+        <v>3.548504476226856</v>
       </c>
       <c r="AX138" t="n">
         <v>1.246443706176061</v>
       </c>
       <c r="AY138" t="n">
-        <v>8731.29255587387</v>
+        <v>8731.296327683798</v>
       </c>
       <c r="AZ138" t="inlineStr"/>
       <c r="BA138" t="n">
@@ -27242,22 +27242,22 @@
         <v>27.5</v>
       </c>
       <c r="AE139" t="n">
-        <v>926.7999877929688</v>
+        <v>910.4000244140625</v>
       </c>
       <c r="AF139" t="n">
-        <v>921.4593237304688</v>
+        <v>923.1197509765625</v>
       </c>
       <c r="AG139" t="n">
-        <v>694.351842956543</v>
+        <v>696.4230020141601</v>
       </c>
       <c r="AH139" t="n">
-        <v>0.005795876090198604</v>
+        <v>-0.01377906447028554</v>
       </c>
       <c r="AI139" t="n">
-        <v>0.33476996884845</v>
+        <v>0.3072515149284969</v>
       </c>
       <c r="AJ139" t="n">
-        <v>0.3270783869556744</v>
+        <v>0.3255158837470349</v>
       </c>
       <c r="AK139" t="n">
         <v>1079</v>
@@ -27266,13 +27266,13 @@
         <v>400.14208984375</v>
       </c>
       <c r="AM139" t="n">
-        <v>-0.1410565451409002</v>
+        <v>-0.1562557697738067</v>
       </c>
       <c r="AN139" t="n">
-        <v>1.316177206339057</v>
+        <v>1.275191856896537</v>
       </c>
       <c r="AO139" t="n">
-        <v>34.94936027490418</v>
+        <v>31.98717739716291</v>
       </c>
       <c r="AP139" t="n">
         <v>107476</v>
@@ -27284,25 +27284,25 @@
         <v>0.6619580571017354</v>
       </c>
       <c r="AS139" t="n">
-        <v>-0.04806901085304904</v>
+        <v>-0.1030541631388546</v>
       </c>
       <c r="AT139" t="n">
-        <v>0.2535817586396945</v>
+        <v>0.214060249351276</v>
       </c>
       <c r="AU139" t="n">
-        <v>0.4853262722247138</v>
+        <v>0.4736287916120494</v>
       </c>
       <c r="AV139" t="n">
-        <v>0.7502039833078895</v>
+        <v>0.8133820500635158</v>
       </c>
       <c r="AW139" t="n">
-        <v>1.971036452042661</v>
+        <v>1.944103461316486</v>
       </c>
       <c r="AX139" t="n">
-        <v>0.6800441544724991</v>
+        <v>0.6503153424621462</v>
       </c>
       <c r="AY139" t="n">
-        <v>314.3192464682254</v>
+        <v>308.7396166912947</v>
       </c>
       <c r="AZ139" t="inlineStr"/>
       <c r="BA139" t="n">
@@ -27638,28 +27638,28 @@
         <v>212.8434069824219</v>
       </c>
       <c r="AG141" t="n">
-        <v>154.8032143783569</v>
+        <v>154.8032144165039</v>
       </c>
       <c r="AH141" t="n">
         <v>0.08774806584251649</v>
       </c>
       <c r="AI141" t="n">
-        <v>0.4955762075236974</v>
+        <v>0.4955762071551537</v>
       </c>
       <c r="AJ141" t="n">
-        <v>0.3749288594370399</v>
+        <v>0.3749288590982265</v>
       </c>
       <c r="AK141" t="n">
         <v>301.7099914550781</v>
       </c>
       <c r="AL141" t="n">
-        <v>84.03205871582031</v>
+        <v>84.03206634521484</v>
       </c>
       <c r="AM141" t="n">
         <v>-0.2326405792665565</v>
       </c>
       <c r="AN141" t="n">
-        <v>1.755139024445604</v>
+        <v>1.755138774302492</v>
       </c>
       <c r="AO141" t="n">
         <v>43.63074780758868</v>
@@ -27680,19 +27680,19 @@
         <v>0.3343589022001288</v>
       </c>
       <c r="AU141" t="n">
-        <v>0.7523533299101399</v>
+        <v>0.7523531275267559</v>
       </c>
       <c r="AV141" t="n">
-        <v>1.509230660718758</v>
+        <v>1.509230453235678</v>
       </c>
       <c r="AW141" t="n">
-        <v>6.81089603857342</v>
+        <v>6.810894530701525</v>
       </c>
       <c r="AX141" t="n">
         <v>0.821280415926525</v>
       </c>
       <c r="AY141" t="n">
-        <v>3814.855705709633</v>
+        <v>3814.853831383067</v>
       </c>
       <c r="AZ141" t="inlineStr"/>
       <c r="BA141" t="n">
@@ -28074,13 +28074,13 @@
         <v>2.276219758479249</v>
       </c>
       <c r="AW143" t="n">
-        <v>2.504804932643056</v>
+        <v>2.50480517328828</v>
       </c>
       <c r="AX143" t="n">
         <v>2.159211975137846</v>
       </c>
       <c r="AY143" t="n">
-        <v>3.026105131180706</v>
+        <v>3.026104178514217</v>
       </c>
       <c r="AZ143" t="inlineStr"/>
       <c r="BA143" t="n">
@@ -28222,28 +28222,28 @@
         <v>380.8338464355469</v>
       </c>
       <c r="AG144" t="n">
-        <v>273.7488339233398</v>
+        <v>273.7488342285156</v>
       </c>
       <c r="AH144" t="n">
         <v>-0.0557561795800755</v>
       </c>
       <c r="AI144" t="n">
-        <v>0.3136129237511838</v>
+        <v>0.313612922286765</v>
       </c>
       <c r="AJ144" t="n">
-        <v>0.3911797941838722</v>
+        <v>0.3911797926329816</v>
       </c>
       <c r="AK144" t="n">
         <v>483.8399963378906</v>
       </c>
       <c r="AL144" t="n">
-        <v>89.91980743408203</v>
+        <v>89.91981506347656</v>
       </c>
       <c r="AM144" t="n">
         <v>-0.2567790822890379</v>
       </c>
       <c r="AN144" t="n">
-        <v>2.999118952374642</v>
+        <v>2.99911861306282</v>
       </c>
       <c r="AO144" t="n">
         <v>39.53668502102783</v>
@@ -28267,16 +28267,16 @@
         <v>0.6637522390864634</v>
       </c>
       <c r="AV144" t="n">
-        <v>2.655653491751345</v>
+        <v>2.655653208220445</v>
       </c>
       <c r="AW144" t="n">
-        <v>1.852877252201813</v>
+        <v>1.852877597557493</v>
       </c>
       <c r="AX144" t="n">
         <v>0.7338900695814854</v>
       </c>
       <c r="AY144" t="n">
-        <v>321.8698005225353</v>
+        <v>321.8699733112988</v>
       </c>
       <c r="AZ144" t="inlineStr"/>
       <c r="BA144" t="n">
@@ -28610,28 +28610,28 @@
         <v>113.3724143981934</v>
       </c>
       <c r="AG146" t="n">
-        <v>85.38335865020753</v>
+        <v>85.3833589553833</v>
       </c>
       <c r="AH146" t="n">
         <v>0.07001335556391641</v>
       </c>
       <c r="AI146" t="n">
-        <v>0.4207686307535397</v>
+        <v>0.4207686256754521</v>
       </c>
       <c r="AJ146" t="n">
-        <v>0.3278045767987343</v>
+        <v>0.3278045720529175</v>
       </c>
       <c r="AK146" t="n">
         <v>129.5154876708984</v>
       </c>
       <c r="AL146" t="n">
-        <v>64.85703277587891</v>
+        <v>64.85704040527344</v>
       </c>
       <c r="AM146" t="n">
         <v>-0.06335528097732224</v>
       </c>
       <c r="AN146" t="n">
-        <v>0.8704216392044128</v>
+        <v>0.8704214191791921</v>
       </c>
       <c r="AO146" t="n">
         <v>53.45739456180635</v>
@@ -28658,13 +28658,13 @@
         <v>0.8007837203613268</v>
       </c>
       <c r="AW146" t="n">
-        <v>1.605746185163595</v>
+        <v>1.605746612192991</v>
       </c>
       <c r="AX146" t="n">
         <v>0.6099895768087134</v>
       </c>
       <c r="AY146" t="n">
-        <v>2447.999423320764</v>
+        <v>2447.998318245272</v>
       </c>
       <c r="AZ146" t="inlineStr"/>
       <c r="BA146" t="n">
@@ -28806,16 +28806,16 @@
         <v>344.7219982910156</v>
       </c>
       <c r="AG147" t="n">
-        <v>193.6150336074829</v>
+        <v>193.6150331878662</v>
       </c>
       <c r="AH147" t="n">
         <v>0.2617993727615253</v>
       </c>
       <c r="AI147" t="n">
-        <v>1.246571421217842</v>
+        <v>1.246571426086776</v>
       </c>
       <c r="AJ147" t="n">
-        <v>0.7804505769416279</v>
+        <v>0.780450580800351</v>
       </c>
       <c r="AK147" t="n">
         <v>465.9599914550781</v>
@@ -28848,19 +28848,19 @@
         <v>1.453969996448112</v>
       </c>
       <c r="AU147" t="n">
-        <v>2.698098364517853</v>
+        <v>2.698098604394358</v>
       </c>
       <c r="AV147" t="n">
         <v>2.452300900624646</v>
       </c>
       <c r="AW147" t="n">
-        <v>8.49142477948886</v>
+        <v>8.491426359621924</v>
       </c>
       <c r="AX147" t="n">
         <v>2.42898800734462</v>
       </c>
       <c r="AY147" t="n">
-        <v>38.61284288930269</v>
+        <v>38.6128463297336</v>
       </c>
       <c r="AZ147" t="inlineStr"/>
       <c r="BA147" t="n">
@@ -29050,13 +29050,13 @@
         <v>0.3509508024738093</v>
       </c>
       <c r="AW148" t="n">
-        <v>1.265500221123102</v>
+        <v>1.265499946928041</v>
       </c>
       <c r="AX148" t="n">
         <v>0.1744469586237913</v>
       </c>
       <c r="AY148" t="n">
-        <v>45.24491761337382</v>
+        <v>45.24490690235807</v>
       </c>
       <c r="AZ148" t="inlineStr"/>
       <c r="BA148" t="n">
@@ -29171,10 +29171,10 @@
         </is>
       </c>
       <c r="Z149" t="n">
-        <v>1.339818000793457</v>
+        <v>1.340141177177429</v>
       </c>
       <c r="AA149" t="n">
-        <v>159578281347.0078</v>
+        <v>159616773091.3311</v>
       </c>
       <c r="AB149" t="inlineStr">
         <is>
@@ -29188,67 +29188,67 @@
         <v>38</v>
       </c>
       <c r="AE149" t="n">
-        <v>1436.400024414062</v>
+        <v>1438.400024414062</v>
       </c>
       <c r="AF149" t="n">
-        <v>1307.171987304687</v>
+        <v>1313.96798828125</v>
       </c>
       <c r="AG149" t="n">
-        <v>1219.082796630859</v>
+        <v>1220.455052490234</v>
       </c>
       <c r="AH149" t="n">
-        <v>0.09886077606041388</v>
+        <v>0.09469944263678531</v>
       </c>
       <c r="AI149" t="n">
-        <v>0.1782628943528659</v>
+        <v>0.1785768115582218</v>
       </c>
       <c r="AJ149" t="n">
-        <v>0.07225857908689837</v>
+        <v>0.07662136807104081</v>
       </c>
       <c r="AK149" t="n">
         <v>1504.199951171875</v>
       </c>
       <c r="AL149" t="n">
-        <v>975.3168334960938</v>
+        <v>977.11669921875</v>
       </c>
       <c r="AM149" t="n">
-        <v>-0.04507374614989967</v>
+        <v>-0.04374413568259317</v>
       </c>
       <c r="AN149" t="n">
-        <v>0.4727522124940495</v>
+        <v>0.4720862160723789</v>
       </c>
       <c r="AO149" t="n">
-        <v>54.26498101929751</v>
+        <v>54.04254798122121</v>
       </c>
       <c r="AP149" t="n">
-        <v>7263301</v>
+        <v>7271649</v>
       </c>
       <c r="AQ149" t="n">
-        <v>28273056.36</v>
+        <v>28273223.32</v>
       </c>
       <c r="AR149" t="n">
-        <v>0.2568983313129151</v>
+        <v>0.2571920759687898</v>
       </c>
       <c r="AS149" t="n">
-        <v>0.1465516989384521</v>
+        <v>0.09969420826763198</v>
       </c>
       <c r="AT149" t="n">
-        <v>0.1335725844535003</v>
+        <v>0.1331835612707564</v>
       </c>
       <c r="AU149" t="n">
-        <v>0.1105242062320975</v>
+        <v>0.1176870197894437</v>
       </c>
       <c r="AV149" t="n">
-        <v>0.4727522124940495</v>
+        <v>0.4559946857814443</v>
       </c>
       <c r="AW149" t="n">
-        <v>14.00565717438729</v>
+        <v>14.36846390410763</v>
       </c>
       <c r="AX149" t="n">
-        <v>0.2000527668804299</v>
+        <v>0.2017236840991483</v>
       </c>
       <c r="AY149" t="n">
-        <v>10.53590605585391</v>
+        <v>10.55196405602961</v>
       </c>
       <c r="AZ149" t="inlineStr"/>
       <c r="BA149" t="n">
@@ -29405,13 +29405,13 @@
         <v>300.0641784667969</v>
       </c>
       <c r="AL150" t="n">
-        <v>150.8650207519531</v>
+        <v>150.8650054931641</v>
       </c>
       <c r="AM150" t="n">
         <v>-0.2085026569531685</v>
       </c>
       <c r="AN150" t="n">
-        <v>0.5742549122138061</v>
+        <v>0.5742550714371035</v>
       </c>
       <c r="AO150" t="n">
         <v>22.26511331067071</v>
@@ -29444,7 +29444,7 @@
         <v>0.05419256041366327</v>
       </c>
       <c r="AY150" t="n">
-        <v>647.3817382215242</v>
+        <v>647.3816327153274</v>
       </c>
       <c r="AZ150" t="inlineStr"/>
       <c r="BA150" t="n">
@@ -29636,7 +29636,7 @@
         <v>0.5667789954459108</v>
       </c>
       <c r="AY151" t="n">
-        <v>7.8961362537878</v>
+        <v>7.89613517248471</v>
       </c>
       <c r="AZ151" t="inlineStr"/>
       <c r="BA151" t="n">
@@ -29822,13 +29822,13 @@
         <v>0.3706422018348623</v>
       </c>
       <c r="AW152" t="n">
-        <v>4.364330746063897</v>
+        <v>4.364331333865288</v>
       </c>
       <c r="AX152" t="n">
         <v>0.348375451263538</v>
       </c>
       <c r="AY152" t="n">
-        <v>17.83057217286446</v>
+        <v>17.83057398364805</v>
       </c>
       <c r="AZ152" t="inlineStr"/>
       <c r="BA152" t="n">
@@ -30014,13 +30014,13 @@
         <v>0.238007897929065</v>
       </c>
       <c r="AW153" t="n">
-        <v>5.212913593236616</v>
+        <v>5.212914102746834</v>
       </c>
       <c r="AX153" t="n">
         <v>-0.03355509631330522</v>
       </c>
       <c r="AY153" t="n">
-        <v>29.10802381311947</v>
+        <v>29.10802680446643</v>
       </c>
       <c r="AZ153" t="inlineStr"/>
       <c r="BA153" t="n">
@@ -30212,7 +30212,7 @@
         <v>0.2543080898858463</v>
       </c>
       <c r="AY154" t="n">
-        <v>-0.1357731724427537</v>
+        <v>-0.1357731035394411</v>
       </c>
       <c r="AZ154" t="inlineStr"/>
       <c r="BA154" t="n">
@@ -30398,13 +30398,13 @@
         <v>1.049789295238969</v>
       </c>
       <c r="AW155" t="n">
-        <v>5.68485230001632</v>
+        <v>5.684852841185671</v>
       </c>
       <c r="AX155" t="n">
         <v>0.157581844149159</v>
       </c>
       <c r="AY155" t="n">
-        <v>59.09308656887164</v>
+        <v>59.09308110238211</v>
       </c>
       <c r="AZ155" t="inlineStr"/>
       <c r="BA155" t="n">
@@ -30988,7 +30988,7 @@
         <v>1.027137855257762</v>
       </c>
       <c r="AY158" t="n">
-        <v>5.736954961447857</v>
+        <v>5.7369558531661</v>
       </c>
       <c r="AZ158" t="inlineStr"/>
       <c r="BA158" t="n">
@@ -31178,7 +31178,7 @@
         <v>0.49674677477929</v>
       </c>
       <c r="AW159" t="n">
-        <v>4.749214113669887</v>
+        <v>4.749214495422165</v>
       </c>
       <c r="AX159" t="n">
         <v>0.3747178990470601</v>
@@ -32612,16 +32612,16 @@
         <v>405.9760382080078</v>
       </c>
       <c r="AG5" t="n">
-        <v>361.2549255371094</v>
+        <v>361.2549252319336</v>
       </c>
       <c r="AH5" t="n">
         <v>-0.0147940676839341</v>
       </c>
       <c r="AI5" t="n">
-        <v>0.1071682984696545</v>
+        <v>0.1071682994049523</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.1237937797094604</v>
+        <v>0.1237937806588028</v>
       </c>
       <c r="AK5" t="n">
         <v>480.8090515136719</v>
@@ -32660,13 +32660,13 @@
         <v>0.4629652450487607</v>
       </c>
       <c r="AW5" t="n">
-        <v>8.384254085964638</v>
+        <v>8.384253246055829</v>
       </c>
       <c r="AX5" t="n">
         <v>0.154834014083173</v>
       </c>
       <c r="AY5" t="n">
-        <v>351.2130314740801</v>
+        <v>351.2129205528598</v>
       </c>
       <c r="AZ5" t="inlineStr"/>
       <c r="BA5" t="n">
@@ -33014,16 +33014,16 @@
         <v>329.1420672607422</v>
       </c>
       <c r="AG7" t="n">
-        <v>227.9347861862183</v>
+        <v>227.9347863006592</v>
       </c>
       <c r="AH7" t="n">
         <v>0.06437317322534364</v>
       </c>
       <c r="AI7" t="n">
-        <v>0.5369746427649391</v>
+        <v>0.5369746419932591</v>
       </c>
       <c r="AJ7" t="n">
-        <v>0.4440185842973505</v>
+        <v>0.4440185835723414</v>
       </c>
       <c r="AK7" t="n">
         <v>433.3299865722656</v>
@@ -33062,13 +33062,13 @@
         <v>2.485740056595084</v>
       </c>
       <c r="AW7" t="n">
-        <v>4.844537693193175</v>
+        <v>4.844538437090752</v>
       </c>
       <c r="AX7" t="n">
         <v>0.8966647974746411</v>
       </c>
       <c r="AY7" t="n">
-        <v>1857.200146520424</v>
+        <v>1857.199852784066</v>
       </c>
       <c r="AZ7" t="inlineStr"/>
       <c r="BA7" t="n">
@@ -33270,7 +33270,7 @@
         <v>1.641861886780454</v>
       </c>
       <c r="AY8" t="n">
-        <v>18.44134625341344</v>
+        <v>18.44135083917955</v>
       </c>
       <c r="AZ8" t="inlineStr"/>
       <c r="BA8" t="n">
@@ -33715,40 +33715,40 @@
         <v>0.8666666666666667</v>
       </c>
       <c r="K2" t="n">
-        <v>0.7273344398567564</v>
+        <v>0.7253525190560661</v>
       </c>
       <c r="L2" t="n">
-        <v>0.6800441544724991</v>
+        <v>0.6503153424621462</v>
       </c>
       <c r="M2" t="n">
-        <v>0.5839277583758825</v>
+        <v>0.583588452388129</v>
       </c>
       <c r="N2" t="n">
-        <v>1.411908074996111</v>
+        <v>1.416119904827568</v>
       </c>
       <c r="O2" t="n">
         <v>1.305639352180217</v>
       </c>
       <c r="P2" t="n">
-        <v>1.231261274528154</v>
+        <v>1.231982266768718</v>
       </c>
       <c r="Q2" t="n">
-        <v>3.982212128027574</v>
+        <v>3.980288208080263</v>
       </c>
       <c r="R2" t="n">
-        <v>3.006203090497208</v>
+        <v>3.006203228329295</v>
       </c>
       <c r="S2" t="n">
-        <v>3.453522603261745</v>
+        <v>3.453212444826061</v>
       </c>
       <c r="T2" t="n">
-        <v>987.015703225061</v>
+        <v>986.643841380923</v>
       </c>
       <c r="U2" t="n">
-        <v>48.65044641518445</v>
+        <v>48.65044226794548</v>
       </c>
       <c r="V2" t="n">
-        <v>1437.128496160032</v>
+        <v>1437.065034929149</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -33766,10 +33766,10 @@
         <v>16</v>
       </c>
       <c r="C3" t="n">
-        <v>1496.124004928353</v>
+        <v>1496.162496672676</v>
       </c>
       <c r="D3" t="n">
-        <v>93.50775030802203</v>
+        <v>93.51015604204223</v>
       </c>
       <c r="E3" t="n">
         <v>47.30320301158594</v>
@@ -33781,7 +33781,7 @@
         <v>85</v>
       </c>
       <c r="H3" t="n">
-        <v>90.48120946802321</v>
+        <v>90.48132572286195</v>
       </c>
       <c r="I3" t="n">
         <v>14</v>
@@ -33790,40 +33790,40 @@
         <v>0.875</v>
       </c>
       <c r="K3" t="n">
-        <v>0.4614154242241409</v>
+        <v>0.4615198565503109</v>
       </c>
       <c r="L3" t="n">
-        <v>0.2271804283831381</v>
+        <v>0.2280158869924973</v>
       </c>
       <c r="M3" t="n">
-        <v>0.8044305441012297</v>
+        <v>0.8045932556116576</v>
       </c>
       <c r="N3" t="n">
-        <v>0.75107079682039</v>
+        <v>0.7500234514008521</v>
       </c>
       <c r="O3" t="n">
         <v>0.5824449702370634</v>
       </c>
       <c r="P3" t="n">
-        <v>1.062701744882527</v>
+        <v>1.060898805341253</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.27399492076843</v>
+        <v>7.296670575950991</v>
       </c>
       <c r="R3" t="n">
-        <v>4.556772429866892</v>
+        <v>4.556772914643727</v>
       </c>
       <c r="S3" t="n">
-        <v>6.185699833358934</v>
+        <v>6.224607212746751</v>
       </c>
       <c r="T3" t="n">
-        <v>247.8259257455878</v>
+        <v>247.8268532057666</v>
       </c>
       <c r="U3" t="n">
-        <v>37.99842177017218</v>
+        <v>37.99842349038764</v>
       </c>
       <c r="V3" t="n">
-        <v>858.2266920626638</v>
+        <v>858.2062360303023</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
@@ -33841,10 +33841,10 @@
         <v>8</v>
       </c>
       <c r="C4" t="n">
-        <v>11972.54559490939</v>
+        <v>11972.66843570861</v>
       </c>
       <c r="D4" t="n">
-        <v>1496.568199363674</v>
+        <v>1496.583554463576</v>
       </c>
       <c r="E4" t="n">
         <v>448.730906624</v>
@@ -33856,7 +33856,7 @@
         <v>85</v>
       </c>
       <c r="H4" t="n">
-        <v>89.70758604960038</v>
+        <v>89.70753774928741</v>
       </c>
       <c r="I4" t="n">
         <v>8</v>
@@ -33865,40 +33865,40 @@
         <v>1</v>
       </c>
       <c r="K4" t="n">
-        <v>0.7956142003891827</v>
+        <v>0.7956141839510227</v>
       </c>
       <c r="L4" t="n">
         <v>0.4358825263117641</v>
       </c>
       <c r="M4" t="n">
-        <v>0.373437047611498</v>
+        <v>0.3734383211174508</v>
       </c>
       <c r="N4" t="n">
-        <v>1.461536661793594</v>
+        <v>1.461536633495111</v>
       </c>
       <c r="O4" t="n">
-        <v>0.8336772562959124</v>
+        <v>0.8336772025518118</v>
       </c>
       <c r="P4" t="n">
-        <v>0.7660153783260093</v>
+        <v>0.766033813408493</v>
       </c>
       <c r="Q4" t="n">
-        <v>5.046953241505195</v>
+        <v>5.046952902772387</v>
       </c>
       <c r="R4" t="n">
         <v>1.531597834322677</v>
       </c>
       <c r="S4" t="n">
-        <v>5.266256114974095</v>
+        <v>5.266375729823522</v>
       </c>
       <c r="T4" t="n">
-        <v>1274.067947302685</v>
+        <v>1274.067782598772</v>
       </c>
       <c r="U4" t="n">
-        <v>368.0056166780973</v>
+        <v>368.0056662041238</v>
       </c>
       <c r="V4" t="n">
-        <v>3689.204468094933</v>
+        <v>3689.166228473247</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
@@ -33940,40 +33940,40 @@
         <v>1</v>
       </c>
       <c r="K5" t="n">
-        <v>2.303326382422048</v>
+        <v>2.281549378431186</v>
       </c>
       <c r="L5" t="n">
         <v>1.841141636730317</v>
       </c>
       <c r="M5" t="n">
-        <v>2.028906411629726</v>
+        <v>2.023149242458056</v>
       </c>
       <c r="N5" t="n">
-        <v>5.03797526641854</v>
+        <v>4.989204617586909</v>
       </c>
       <c r="O5" t="n">
         <v>5.429883716020687</v>
       </c>
       <c r="P5" t="n">
-        <v>4.582935046181752</v>
+        <v>4.570041600597397</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.606826823379718</v>
+        <v>5.593319177576054</v>
       </c>
       <c r="R5" t="n">
         <v>5.771676410395915</v>
       </c>
       <c r="S5" t="n">
-        <v>6.323647196347297</v>
+        <v>6.320076178753674</v>
       </c>
       <c r="T5" t="n">
-        <v>35.10414900302618</v>
+        <v>35.04190478791755</v>
       </c>
       <c r="U5" t="n">
-        <v>28.33033194284154</v>
+        <v>28.33032159671425</v>
       </c>
       <c r="V5" t="n">
-        <v>48.2469449782201</v>
+        <v>48.23049466471921</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
@@ -33991,10 +33991,10 @@
         <v>23</v>
       </c>
       <c r="C6" t="n">
-        <v>1750.926637813314</v>
+        <v>1750.923699612769</v>
       </c>
       <c r="D6" t="n">
-        <v>76.12724512231799</v>
+        <v>76.12711737446823</v>
       </c>
       <c r="E6" t="n">
         <v>43.22962687916699</v>
@@ -34006,7 +34006,7 @@
         <v>85</v>
       </c>
       <c r="H6" t="n">
-        <v>88.63419468922891</v>
+        <v>88.63431825373999</v>
       </c>
       <c r="I6" t="n">
         <v>20</v>
@@ -34015,40 +34015,40 @@
         <v>0.8695652173913043</v>
       </c>
       <c r="K6" t="n">
-        <v>0.5210620311618787</v>
+        <v>0.5200356810245045</v>
       </c>
       <c r="L6" t="n">
         <v>0.4983397216186964</v>
       </c>
       <c r="M6" t="n">
-        <v>0.5390307555256388</v>
+        <v>0.5373625032870161</v>
       </c>
       <c r="N6" t="n">
-        <v>1.002775391335191</v>
+        <v>1.005412930331974</v>
       </c>
       <c r="O6" t="n">
-        <v>0.6849127815543512</v>
+        <v>0.6849127996371749</v>
       </c>
       <c r="P6" t="n">
-        <v>0.8597937437412457</v>
+        <v>0.8624194491710256</v>
       </c>
       <c r="Q6" t="n">
-        <v>3.118208769985672</v>
+        <v>3.109227775740857</v>
       </c>
       <c r="R6" t="n">
-        <v>1.622946079240163</v>
+        <v>1.622945966184871</v>
       </c>
       <c r="S6" t="n">
-        <v>2.896820324421084</v>
+        <v>2.887392977911969</v>
       </c>
       <c r="T6" t="n">
-        <v>175.1181854964813</v>
+        <v>175.1153744367016</v>
       </c>
       <c r="U6" t="n">
-        <v>31.08766645380388</v>
+        <v>31.0876695332767</v>
       </c>
       <c r="V6" t="n">
-        <v>336.5079937325692</v>
+        <v>336.5046055009283</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
@@ -34066,10 +34066,10 @@
         <v>13</v>
       </c>
       <c r="C7" t="n">
-        <v>4886.694706455062</v>
+        <v>4886.4359943285</v>
       </c>
       <c r="D7" t="n">
-        <v>407.2245588712552</v>
+        <v>407.202999527375</v>
       </c>
       <c r="E7" t="n">
         <v>232.3807105032109</v>
@@ -34081,7 +34081,7 @@
         <v>85</v>
       </c>
       <c r="H7" t="n">
-        <v>85.33438429557582</v>
+        <v>85.33440199953682</v>
       </c>
       <c r="I7" t="n">
         <v>12</v>
@@ -34090,40 +34090,40 @@
         <v>0.9230769230769231</v>
       </c>
       <c r="K7" t="n">
-        <v>2.105832567555217</v>
+        <v>2.105832592616566</v>
       </c>
       <c r="L7" t="n">
         <v>1.664310437762967</v>
       </c>
       <c r="M7" t="n">
-        <v>2.190735940288443</v>
+        <v>2.190763210442809</v>
       </c>
       <c r="N7" t="n">
-        <v>9.886561599551063</v>
+        <v>9.886561620166002</v>
       </c>
       <c r="O7" t="n">
-        <v>6.732196413259947</v>
+        <v>6.732196257695808</v>
       </c>
       <c r="P7" t="n">
-        <v>8.704597341596575</v>
+        <v>8.704791764428737</v>
       </c>
       <c r="Q7" t="n">
-        <v>7.412159889257294</v>
+        <v>7.412160262351141</v>
       </c>
       <c r="R7" t="n">
-        <v>5.096490814723951</v>
+        <v>5.096490694560895</v>
       </c>
       <c r="S7" t="n">
-        <v>9.726786369303451</v>
+        <v>9.72677353701183</v>
       </c>
       <c r="T7" t="n">
-        <v>329.9796135730608</v>
+        <v>329.979581322507</v>
       </c>
       <c r="U7" t="n">
         <v>58.94978088356092</v>
       </c>
       <c r="V7" t="n">
-        <v>394.0965509432351</v>
+        <v>394.1157227797556</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
@@ -34165,40 +34165,40 @@
         <v>0.75</v>
       </c>
       <c r="K8" t="n">
-        <v>0.2611099799062427</v>
+        <v>0.2609476375450241</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1987162444835392</v>
+        <v>0.1967042620419301</v>
       </c>
       <c r="M8" t="n">
-        <v>0.1627585029045427</v>
+        <v>0.160815145947719</v>
       </c>
       <c r="N8" t="n">
-        <v>0.3153085004829326</v>
+        <v>0.3460367117614402</v>
       </c>
       <c r="O8" t="n">
-        <v>0.2221291571549595</v>
+        <v>0.2277517241939561</v>
       </c>
       <c r="P8" t="n">
-        <v>0.1904252267567244</v>
+        <v>0.2020411536850994</v>
       </c>
       <c r="Q8" t="n">
-        <v>1.620702308913479</v>
+        <v>1.614975501118781</v>
       </c>
       <c r="R8" t="n">
-        <v>1.576368462334159</v>
+        <v>1.541523208624256</v>
       </c>
       <c r="S8" t="n">
-        <v>1.389659618635162</v>
+        <v>1.355407295924796</v>
       </c>
       <c r="T8" t="n">
-        <v>98.61344081515855</v>
+        <v>98.6478183584028</v>
       </c>
       <c r="U8" t="n">
-        <v>87.78331744073463</v>
+        <v>87.90204016383107</v>
       </c>
       <c r="V8" t="n">
-        <v>76.02879389579181</v>
+        <v>75.98837766026236</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
@@ -34216,10 +34216,10 @@
         <v>21</v>
       </c>
       <c r="C9" t="n">
-        <v>3639.364546616234</v>
+        <v>3639.66375538361</v>
       </c>
       <c r="D9" t="n">
-        <v>173.3030736483921</v>
+        <v>173.3173216849338</v>
       </c>
       <c r="E9" t="n">
         <v>63.484960768</v>
@@ -34231,7 +34231,7 @@
         <v>85</v>
       </c>
       <c r="H9" t="n">
-        <v>83.82058521833815</v>
+        <v>83.82091624059321</v>
       </c>
       <c r="I9" t="n">
         <v>17</v>
@@ -34240,40 +34240,40 @@
         <v>0.8095238095238095</v>
       </c>
       <c r="K9" t="n">
-        <v>0.723236616641208</v>
+        <v>0.7227161366391155</v>
       </c>
       <c r="L9" t="n">
         <v>0.7195215682835878</v>
       </c>
       <c r="M9" t="n">
-        <v>0.4569560371075359</v>
+        <v>0.4567927085220017</v>
       </c>
       <c r="N9" t="n">
-        <v>2.346580830523993</v>
+        <v>2.346930810111189</v>
       </c>
       <c r="O9" t="n">
         <v>1.649707124257812</v>
       </c>
       <c r="P9" t="n">
-        <v>1.513633691248002</v>
+        <v>1.513834657166214</v>
       </c>
       <c r="Q9" t="n">
-        <v>7.927923568162472</v>
+        <v>7.923259258574319</v>
       </c>
       <c r="R9" t="n">
-        <v>3.757894722428535</v>
+        <v>3.757894179517444</v>
       </c>
       <c r="S9" t="n">
-        <v>9.39246567419897</v>
+        <v>9.393711037368867</v>
       </c>
       <c r="T9" t="n">
-        <v>193.3861672047686</v>
+        <v>193.3786416433888</v>
       </c>
       <c r="U9" t="n">
-        <v>26.81621423939938</v>
+        <v>26.72739497324481</v>
       </c>
       <c r="V9" t="n">
-        <v>310.9244825403918</v>
+        <v>310.9161614111101</v>
       </c>
       <c r="W9" t="inlineStr">
         <is>
@@ -34315,13 +34315,13 @@
         <v>0.5</v>
       </c>
       <c r="K10" t="n">
-        <v>0.2102573472522999</v>
+        <v>0.2102573578523762</v>
       </c>
       <c r="L10" t="n">
         <v>0.09311950856431284</v>
       </c>
       <c r="M10" t="n">
-        <v>0.2520480258477386</v>
+        <v>0.2520480357927934</v>
       </c>
       <c r="N10" t="n">
         <v>0.2458892035961248</v>
@@ -34333,22 +34333,22 @@
         <v>0.4432512953737321</v>
       </c>
       <c r="Q10" t="n">
-        <v>1.646266112248328</v>
+        <v>1.646266232450466</v>
       </c>
       <c r="R10" t="n">
         <v>0.7604729894282652</v>
       </c>
       <c r="S10" t="n">
-        <v>6.253500885573207</v>
+        <v>6.253501474352138</v>
       </c>
       <c r="T10" t="n">
-        <v>61.6433730625065</v>
+        <v>61.64337716404984</v>
       </c>
       <c r="U10" t="n">
         <v>7.762627632492336</v>
       </c>
       <c r="V10" t="n">
-        <v>254.9729418945152</v>
+        <v>254.9729038340867</v>
       </c>
       <c r="W10" t="inlineStr">
         <is>
@@ -34399,31 +34399,31 @@
         <v>1.52461168451704</v>
       </c>
       <c r="N11" t="n">
-        <v>0.2150646302695592</v>
+        <v>0.2150647570185179</v>
       </c>
       <c r="O11" t="n">
-        <v>0.2150646302695592</v>
+        <v>0.2150647570185179</v>
       </c>
       <c r="P11" t="n">
-        <v>1.088979265447312</v>
+        <v>1.088979507089518</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.001995282711361</v>
+        <v>1.001995068756024</v>
       </c>
       <c r="R11" t="n">
-        <v>1.001995282711361</v>
+        <v>1.001995068756024</v>
       </c>
       <c r="S11" t="n">
-        <v>1.001995282711361</v>
+        <v>1.001995068756024</v>
       </c>
       <c r="T11" t="n">
-        <v>15.76681283666081</v>
+        <v>15.76681816677099</v>
       </c>
       <c r="U11" t="n">
-        <v>15.76681283666081</v>
+        <v>15.76681816677099</v>
       </c>
       <c r="V11" t="n">
-        <v>30.15075386699116</v>
+        <v>30.15076402864925</v>
       </c>
       <c r="W11" t="inlineStr">
         <is>
@@ -34465,40 +34465,40 @@
         <v>0.2105263157894737</v>
       </c>
       <c r="K12" t="n">
-        <v>0.01168974001694152</v>
+        <v>0.009916394939796638</v>
       </c>
       <c r="L12" t="n">
         <v>0.02155212588028221</v>
       </c>
       <c r="M12" t="n">
-        <v>0.1941747190447664</v>
+        <v>0.1902767800191833</v>
       </c>
       <c r="N12" t="n">
-        <v>0.2532544291639344</v>
+        <v>0.2505360673819916</v>
       </c>
       <c r="O12" t="n">
         <v>0.2522044132542418</v>
       </c>
       <c r="P12" t="n">
-        <v>0.4030073905286187</v>
+        <v>0.3970322874329167</v>
       </c>
       <c r="Q12" t="n">
-        <v>2.492409329334427</v>
+        <v>2.473428030958024</v>
       </c>
       <c r="R12" t="n">
-        <v>1.699661016949153</v>
+        <v>1.699660533643547</v>
       </c>
       <c r="S12" t="n">
-        <v>2.291578248968016</v>
+        <v>2.243072145301392</v>
       </c>
       <c r="T12" t="n">
-        <v>78.00173570356627</v>
+        <v>77.99177181410191</v>
       </c>
       <c r="U12" t="n">
-        <v>13.01174408365016</v>
+        <v>13.01174290504081</v>
       </c>
       <c r="V12" t="n">
-        <v>108.6302089828917</v>
+        <v>108.6083264718735</v>
       </c>
       <c r="W12" t="inlineStr">
         <is>
@@ -34540,13 +34540,13 @@
         <v>0.3333333333333333</v>
       </c>
       <c r="K13" t="n">
-        <v>0.5548069150076028</v>
+        <v>0.5548069289366998</v>
       </c>
       <c r="L13" t="n">
         <v>0.05695954192774511</v>
       </c>
       <c r="M13" t="n">
-        <v>0.01272236499219526</v>
+        <v>0.01272240383025292</v>
       </c>
       <c r="N13" t="n">
         <v>0.7305351261040899</v>
@@ -34558,22 +34558,22 @@
         <v>0.3106504585193416</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.5024626683807663</v>
+        <v>0.5024626815934734</v>
       </c>
       <c r="R13" t="n">
-        <v>0.421402410238742</v>
+        <v>0.4214024930006172</v>
       </c>
       <c r="S13" t="n">
-        <v>0.9555870704686314</v>
+        <v>0.9555871230072505</v>
       </c>
       <c r="T13" t="n">
-        <v>1054.194266907383</v>
+        <v>1054.194391575702</v>
       </c>
       <c r="U13" t="n">
-        <v>13.32053004241692</v>
+        <v>13.32052915366983</v>
       </c>
       <c r="V13" t="n">
-        <v>2114.389039377671</v>
+        <v>2114.389480019465</v>
       </c>
       <c r="W13" t="inlineStr">
         <is>
@@ -34624,31 +34624,31 @@
         <v>-0.0511859355338434</v>
       </c>
       <c r="N14" t="n">
-        <v>0.3715001660228982</v>
+        <v>0.3715001416727851</v>
       </c>
       <c r="O14" t="n">
         <v>0.08879809751909096</v>
       </c>
       <c r="P14" t="n">
-        <v>0.2403582871187377</v>
+        <v>0.2403582566820559</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.5256373482043928</v>
+        <v>0.5256374271316632</v>
       </c>
       <c r="R14" t="n">
-        <v>0.4364418153609975</v>
+        <v>0.436441943995166</v>
       </c>
       <c r="S14" t="n">
-        <v>0.6773288453664682</v>
+        <v>0.6773289300522866</v>
       </c>
       <c r="T14" t="n">
-        <v>16.36577907330306</v>
+        <v>16.36577750168141</v>
       </c>
       <c r="U14" t="n">
-        <v>3.138295244484146</v>
+        <v>3.138295688045482</v>
       </c>
       <c r="V14" t="n">
-        <v>2.869338379592058</v>
+        <v>2.869338172427715</v>
       </c>
       <c r="W14" t="inlineStr">
         <is>

</xml_diff>